<commit_message>
rerun model phi4:14b plain GOT results generated
</commit_message>
<xml_diff>
--- a/results/phi4_14b/comparison_GoTPlainLLM/GoTPlainLLM_consolidated.xlsx
+++ b/results/phi4_14b/comparison_GoTPlainLLM/GoTPlainLLM_consolidated.xlsx
@@ -545,47 +545,49 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.01010100960871342</v>
+        <v>0.2201257813921523</v>
       </c>
       <c r="D2" t="n">
-        <v>7.188271943170174e-260</v>
+        <v>2.027317064172704e-155</v>
       </c>
       <c r="E2" t="n">
-        <v>0.3382570147514343</v>
+        <v>0.6062899231910706</v>
       </c>
       <c r="F2" t="n">
-        <v>12.42500000000001</v>
+        <v>16.45019067796611</v>
       </c>
       <c r="G2" t="n">
-        <v>0.06717123935666983</v>
+        <v>0.6877956480605487</v>
       </c>
       <c r="H2" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="I2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J2" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J2" t="n">
+        <v>1</v>
+      </c>
       <c r="K2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L2" t="n">
         <v>0</v>
       </c>
       <c r="M2" t="n">
-        <v>0.1111111111111111</v>
+        <v>0.3069306930693069</v>
       </c>
       <c r="N2" t="n">
-        <v>0.003021955490112305</v>
+        <v>22.12478852272034</v>
       </c>
       <c r="O2" t="n">
-        <v>1122.52734375</v>
+        <v>1125.8359375</v>
       </c>
       <c r="P2" t="n">
-        <v>11.7</v>
+        <v>11.9</v>
       </c>
       <c r="Q2" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R2" t="n">
         <v>0</v>
@@ -594,7 +596,7 @@
         <v>0</v>
       </c>
       <c r="T2" t="n">
-        <v>0.003018617630004883</v>
+        <v>22.12478542327881</v>
       </c>
       <c r="U2" t="n">
         <v>0</v>
@@ -610,47 +612,49 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0</v>
+        <v>0.08333333146701394</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>8.087494814426946e-232</v>
       </c>
       <c r="E3" t="n">
-        <v>0.3607856035232544</v>
+        <v>0.4632394313812256</v>
       </c>
       <c r="F3" t="n">
-        <v>12.42500000000001</v>
+        <v>39.02767581475129</v>
       </c>
       <c r="G3" t="n">
-        <v>0.6513761467889908</v>
+        <v>4.275229357798165</v>
       </c>
       <c r="H3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I3" t="n">
         <v>0</v>
       </c>
-      <c r="J3" t="inlineStr"/>
+      <c r="J3" t="n">
+        <v>1</v>
+      </c>
       <c r="K3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L3" t="n">
         <v>0</v>
       </c>
       <c r="M3" t="n">
-        <v>0.1111111111111111</v>
+        <v>0.2307692307692308</v>
       </c>
       <c r="N3" t="n">
-        <v>0.001966238021850586</v>
+        <v>19.10640835762024</v>
       </c>
       <c r="O3" t="n">
-        <v>1122.53515625</v>
+        <v>1125.9140625</v>
       </c>
       <c r="P3" t="n">
-        <v>0</v>
+        <v>10.7</v>
       </c>
       <c r="Q3" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R3" t="n">
         <v>0</v>
@@ -659,7 +663,7 @@
         <v>0</v>
       </c>
       <c r="T3" t="n">
-        <v>0.001963376998901367</v>
+        <v>19.10640573501587</v>
       </c>
       <c r="U3" t="n">
         <v>0</v>
@@ -675,47 +679,49 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0</v>
+        <v>0.2194092782011431</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>2.853552648457251e-156</v>
       </c>
       <c r="E4" t="n">
-        <v>0.2861286401748657</v>
+        <v>0.5087727904319763</v>
       </c>
       <c r="F4" t="n">
-        <v>12.42500000000001</v>
+        <v>27.79104591836736</v>
       </c>
       <c r="G4" t="n">
-        <v>0.07585470085470085</v>
+        <v>0.4636752136752137</v>
       </c>
       <c r="H4" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="I4" t="n">
         <v>1</v>
       </c>
-      <c r="J4" t="inlineStr"/>
+      <c r="J4" t="n">
+        <v>1</v>
+      </c>
       <c r="K4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L4" t="n">
         <v>0</v>
       </c>
       <c r="M4" t="n">
-        <v>0.1111111111111111</v>
+        <v>0.1666666666666667</v>
       </c>
       <c r="N4" t="n">
-        <v>0.002119302749633789</v>
+        <v>17.32344770431519</v>
       </c>
       <c r="O4" t="n">
-        <v>1122.53515625</v>
+        <v>1125.953125</v>
       </c>
       <c r="P4" t="n">
-        <v>0</v>
+        <v>11.9</v>
       </c>
       <c r="Q4" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R4" t="n">
         <v>0</v>
@@ -724,7 +730,7 @@
         <v>0</v>
       </c>
       <c r="T4" t="n">
-        <v>0.002118110656738281</v>
+        <v>17.32344579696655</v>
       </c>
       <c r="U4" t="n">
         <v>0</v>
@@ -740,47 +746,49 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0</v>
+        <v>0.2471264320869666</v>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>0.01747257096087728</v>
       </c>
       <c r="E5" t="n">
-        <v>0.2819922566413879</v>
+        <v>0.5634866952896118</v>
       </c>
       <c r="F5" t="n">
-        <v>12.42500000000001</v>
+        <v>39.7559782608696</v>
       </c>
       <c r="G5" t="n">
-        <v>0.05810147299509002</v>
+        <v>0.5973813420621932</v>
       </c>
       <c r="H5" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="I5" t="n">
         <v>1</v>
       </c>
-      <c r="J5" t="inlineStr"/>
+      <c r="J5" t="n">
+        <v>1</v>
+      </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="L5" t="n">
         <v>0</v>
       </c>
       <c r="M5" t="n">
-        <v>0.1111111111111111</v>
+        <v>0.25</v>
       </c>
       <c r="N5" t="n">
-        <v>0.001869916915893555</v>
+        <v>20.01042413711548</v>
       </c>
       <c r="O5" t="n">
-        <v>1122.53515625</v>
+        <v>1127.4765625</v>
       </c>
       <c r="P5" t="n">
-        <v>0</v>
+        <v>10.6</v>
       </c>
       <c r="Q5" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R5" t="n">
         <v>0</v>
@@ -789,7 +797,7 @@
         <v>0</v>
       </c>
       <c r="T5" t="n">
-        <v>0.001868486404418945</v>
+        <v>20.01042199134827</v>
       </c>
       <c r="U5" t="n">
         <v>0</v>
@@ -805,47 +813,49 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.01273885288652687</v>
+        <v>0.2330827018689582</v>
       </c>
       <c r="D6" t="n">
-        <v>7.842246496009318e-255</v>
+        <v>1.874738583366479e-155</v>
       </c>
       <c r="E6" t="n">
-        <v>0.3198220431804657</v>
+        <v>0.559995710849762</v>
       </c>
       <c r="F6" t="n">
-        <v>12.42500000000001</v>
+        <v>23.97508960573478</v>
       </c>
       <c r="G6" t="n">
-        <v>0.08160919540229886</v>
+        <v>0.7091954022988506</v>
       </c>
       <c r="H6" t="n">
-        <v>0</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="I6" t="n">
         <v>1</v>
       </c>
-      <c r="J6" t="inlineStr"/>
+      <c r="J6" t="n">
+        <v>1</v>
+      </c>
       <c r="K6" t="n">
-        <v>0</v>
+        <v>0.85</v>
       </c>
       <c r="L6" t="n">
         <v>0</v>
       </c>
       <c r="M6" t="n">
-        <v>0.1111111111111111</v>
+        <v>0.2045454545454545</v>
       </c>
       <c r="N6" t="n">
-        <v>0.002080678939819336</v>
+        <v>21.75261282920837</v>
       </c>
       <c r="O6" t="n">
-        <v>1122.53515625</v>
+        <v>1127.55078125</v>
       </c>
       <c r="P6" t="n">
-        <v>25</v>
+        <v>11.8</v>
       </c>
       <c r="Q6" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R6" t="n">
         <v>0</v>
@@ -854,7 +864,7 @@
         <v>0</v>
       </c>
       <c r="T6" t="n">
-        <v>0.002079486846923828</v>
+        <v>21.75261068344116</v>
       </c>
       <c r="U6" t="n">
         <v>0</v>
@@ -870,47 +880,49 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.004032257864935623</v>
+        <v>0.1618886986692981</v>
       </c>
       <c r="D7" t="n">
-        <v>0</v>
+        <v>3.528448916709317e-82</v>
       </c>
       <c r="E7" t="n">
-        <v>0.3422526717185974</v>
+        <v>0.5546762943267822</v>
       </c>
       <c r="F7" t="n">
-        <v>12.42500000000001</v>
+        <v>16.54755528255532</v>
       </c>
       <c r="G7" t="n">
-        <v>0.02065755018911842</v>
+        <v>0.1786441664242072</v>
       </c>
       <c r="H7" t="n">
         <v>0</v>
       </c>
       <c r="I7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J7" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J7" t="n">
+        <v>1</v>
+      </c>
       <c r="K7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L7" t="n">
         <v>0</v>
       </c>
       <c r="M7" t="n">
-        <v>0.1428571428571428</v>
+        <v>0.2682926829268293</v>
       </c>
       <c r="N7" t="n">
-        <v>0.002376794815063477</v>
+        <v>31.42953681945801</v>
       </c>
       <c r="O7" t="n">
-        <v>1122.640625</v>
+        <v>1127.90234375</v>
       </c>
       <c r="P7" t="n">
-        <v>0</v>
+        <v>10.8</v>
       </c>
       <c r="Q7" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R7" t="n">
         <v>0</v>
@@ -919,7 +931,7 @@
         <v>0</v>
       </c>
       <c r="T7" t="n">
-        <v>0.002375364303588867</v>
+        <v>31.4295346736908</v>
       </c>
       <c r="U7" t="n">
         <v>0</v>
@@ -935,47 +947,49 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0</v>
+        <v>0.205714281172898</v>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>8.952333798159982e-156</v>
       </c>
       <c r="E8" t="n">
-        <v>0.3306046426296234</v>
+        <v>0.6030941605567932</v>
       </c>
       <c r="F8" t="n">
-        <v>12.42500000000001</v>
+        <v>23.47012983425415</v>
       </c>
       <c r="G8" t="n">
-        <v>0.04930555555555555</v>
+        <v>0.48125</v>
       </c>
       <c r="H8" t="n">
-        <v>0</v>
+        <v>0.15</v>
       </c>
       <c r="I8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J8" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J8" t="n">
+        <v>1</v>
+      </c>
       <c r="K8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L8" t="n">
         <v>0</v>
       </c>
       <c r="M8" t="n">
-        <v>0.05882352941176471</v>
+        <v>0.1525423728813559</v>
       </c>
       <c r="N8" t="n">
-        <v>0.002924680709838867</v>
+        <v>29.44839692115784</v>
       </c>
       <c r="O8" t="n">
-        <v>1122.66796875</v>
+        <v>1127.90234375</v>
       </c>
       <c r="P8" t="n">
-        <v>20</v>
+        <v>11.5</v>
       </c>
       <c r="Q8" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R8" t="n">
         <v>0</v>
@@ -984,7 +998,7 @@
         <v>0</v>
       </c>
       <c r="T8" t="n">
-        <v>0.002910852432250977</v>
+        <v>29.44839525222778</v>
       </c>
       <c r="U8" t="n">
         <v>0</v>
@@ -1000,27 +1014,29 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.006993006649469429</v>
+        <v>0.1719901677153501</v>
       </c>
       <c r="D9" t="n">
-        <v>4.626996437597695e-283</v>
+        <v>3.879804140492458e-156</v>
       </c>
       <c r="E9" t="n">
-        <v>0.3232488930225372</v>
+        <v>0.5681236386299133</v>
       </c>
       <c r="F9" t="n">
-        <v>12.42500000000001</v>
+        <v>35.69700980392159</v>
       </c>
       <c r="G9" t="n">
-        <v>0.04113557358053303</v>
+        <v>0.3951332560834299</v>
       </c>
       <c r="H9" t="n">
-        <v>0</v>
+        <v>0.3125</v>
       </c>
       <c r="I9" t="n">
         <v>1</v>
       </c>
-      <c r="J9" t="inlineStr"/>
+      <c r="J9" t="n">
+        <v>1</v>
+      </c>
       <c r="K9" t="n">
         <v>0</v>
       </c>
@@ -1028,19 +1044,19 @@
         <v>0</v>
       </c>
       <c r="M9" t="n">
-        <v>0.1111111111111111</v>
+        <v>0.1780821917808219</v>
       </c>
       <c r="N9" t="n">
-        <v>0.001907587051391602</v>
+        <v>29.57351756095886</v>
       </c>
       <c r="O9" t="n">
-        <v>1122.66796875</v>
+        <v>1127.90234375</v>
       </c>
       <c r="P9" t="n">
-        <v>0</v>
+        <v>11.2</v>
       </c>
       <c r="Q9" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R9" t="n">
         <v>0</v>
@@ -1049,7 +1065,7 @@
         <v>0</v>
       </c>
       <c r="T9" t="n">
-        <v>0.001906633377075195</v>
+        <v>29.57351541519165</v>
       </c>
       <c r="U9" t="n">
         <v>0</v>
@@ -1065,47 +1081,49 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0</v>
+        <v>0.1041666638428338</v>
       </c>
       <c r="D10" t="n">
-        <v>0</v>
+        <v>1.396161808312207e-235</v>
       </c>
       <c r="E10" t="n">
-        <v>0.3218375742435455</v>
+        <v>0.5290889739990234</v>
       </c>
       <c r="F10" t="n">
-        <v>12.42500000000001</v>
+        <v>13.94900000000001</v>
       </c>
       <c r="G10" t="n">
-        <v>0.04695767195767196</v>
+        <v>0.1858465608465608</v>
       </c>
       <c r="H10" t="n">
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="I10" t="n">
         <v>0</v>
       </c>
-      <c r="J10" t="inlineStr"/>
+      <c r="J10" t="n">
+        <v>1</v>
+      </c>
       <c r="K10" t="n">
-        <v>0</v>
+        <v>0.75</v>
       </c>
       <c r="L10" t="n">
         <v>0</v>
       </c>
       <c r="M10" t="n">
-        <v>0.05882352941176471</v>
+        <v>0.07216494845360824</v>
       </c>
       <c r="N10" t="n">
-        <v>0.002264976501464844</v>
+        <v>26.87655830383301</v>
       </c>
       <c r="O10" t="n">
-        <v>1122.66796875</v>
+        <v>1127.90234375</v>
       </c>
       <c r="P10" t="n">
-        <v>25</v>
+        <v>11.2</v>
       </c>
       <c r="Q10" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R10" t="n">
         <v>0</v>
@@ -1114,7 +1132,7 @@
         <v>0</v>
       </c>
       <c r="T10" t="n">
-        <v>0.002264022827148438</v>
+        <v>26.8765561580658</v>
       </c>
       <c r="U10" t="n">
         <v>0</v>
@@ -1130,47 +1148,49 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.006756756424625656</v>
+        <v>0.1557177574227007</v>
       </c>
       <c r="D11" t="n">
-        <v>3.199290466293744e-295</v>
+        <v>2.666523432317515e-80</v>
       </c>
       <c r="E11" t="n">
-        <v>0.3080631196498871</v>
+        <v>0.5482152104377747</v>
       </c>
       <c r="F11" t="n">
-        <v>12.42500000000001</v>
+        <v>29.03810071574645</v>
       </c>
       <c r="G11" t="n">
-        <v>0.03881902679059596</v>
+        <v>0.3603061782394751</v>
       </c>
       <c r="H11" t="n">
-        <v>0</v>
+        <v>0.2222222222222222</v>
       </c>
       <c r="I11" t="n">
         <v>1</v>
       </c>
-      <c r="J11" t="inlineStr"/>
+      <c r="J11" t="n">
+        <v>1</v>
+      </c>
       <c r="K11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L11" t="n">
         <v>0</v>
       </c>
       <c r="M11" t="n">
-        <v>0.1111111111111111</v>
+        <v>0.2</v>
       </c>
       <c r="N11" t="n">
-        <v>0.00187373161315918</v>
+        <v>28.06247925758362</v>
       </c>
       <c r="O11" t="n">
-        <v>1122.66796875</v>
+        <v>1127.9375</v>
       </c>
       <c r="P11" t="n">
-        <v>0</v>
+        <v>10.6</v>
       </c>
       <c r="Q11" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R11" t="n">
         <v>0</v>
@@ -1179,7 +1199,7 @@
         <v>0</v>
       </c>
       <c r="T11" t="n">
-        <v>0.001872539520263672</v>
+        <v>28.06247735023499</v>
       </c>
       <c r="U11" t="n">
         <v>0</v>
@@ -1195,47 +1215,49 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0</v>
+        <v>0.1975308599489103</v>
       </c>
       <c r="D12" t="n">
-        <v>0</v>
+        <v>0.003872628873636948</v>
       </c>
       <c r="E12" t="n">
-        <v>0.3184725940227509</v>
+        <v>0.6138515472412109</v>
       </c>
       <c r="F12" t="n">
-        <v>12.42500000000001</v>
+        <v>38.22492549335482</v>
       </c>
       <c r="G12" t="n">
-        <v>0.04043280182232346</v>
+        <v>0.3997722095671982</v>
       </c>
       <c r="H12" t="n">
-        <v>0</v>
+        <v>0.1111111111111111</v>
       </c>
       <c r="I12" t="n">
-        <v>0</v>
-      </c>
-      <c r="J12" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J12" t="n">
+        <v>1</v>
+      </c>
       <c r="K12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L12" t="n">
         <v>0</v>
       </c>
       <c r="M12" t="n">
-        <v>0.05882352941176471</v>
+        <v>0.1379310344827586</v>
       </c>
       <c r="N12" t="n">
-        <v>0.002344369888305664</v>
+        <v>26.51732444763184</v>
       </c>
       <c r="O12" t="n">
-        <v>1122.66796875</v>
+        <v>1127.953125</v>
       </c>
       <c r="P12" t="n">
-        <v>0</v>
+        <v>11.3</v>
       </c>
       <c r="Q12" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R12" t="n">
         <v>0</v>
@@ -1244,7 +1266,7 @@
         <v>0</v>
       </c>
       <c r="T12" t="n">
-        <v>0.002343416213989258</v>
+        <v>26.51732277870178</v>
       </c>
       <c r="U12" t="n">
         <v>0</v>
@@ -1260,47 +1282,49 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>0.006644517945718055</v>
+        <v>0.3239436577310499</v>
       </c>
       <c r="D13" t="n">
-        <v>1.737745674680046e-291</v>
+        <v>0.03848960639779165</v>
       </c>
       <c r="E13" t="n">
-        <v>0.326636791229248</v>
+        <v>0.5766304731369019</v>
       </c>
       <c r="F13" t="n">
-        <v>12.42500000000001</v>
+        <v>53.01235172413797</v>
       </c>
       <c r="G13" t="n">
-        <v>0.0393569844789357</v>
+        <v>0.4235033259423504</v>
       </c>
       <c r="H13" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="I13" t="n">
         <v>1</v>
       </c>
-      <c r="J13" t="inlineStr"/>
+      <c r="J13" t="n">
+        <v>1</v>
+      </c>
       <c r="K13" t="n">
-        <v>0</v>
+        <v>0.75</v>
       </c>
       <c r="L13" t="n">
         <v>0</v>
       </c>
       <c r="M13" t="n">
-        <v>0.1111111111111111</v>
+        <v>0.4214876033057851</v>
       </c>
       <c r="N13" t="n">
-        <v>0.002075910568237305</v>
+        <v>22.90320491790771</v>
       </c>
       <c r="O13" t="n">
-        <v>1122.66796875</v>
+        <v>1127.953125</v>
       </c>
       <c r="P13" t="n">
-        <v>25</v>
+        <v>11.6</v>
       </c>
       <c r="Q13" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R13" t="n">
         <v>0</v>
@@ -1309,7 +1333,7 @@
         <v>0</v>
       </c>
       <c r="T13" t="n">
-        <v>0.002074480056762695</v>
+        <v>22.90320301055908</v>
       </c>
       <c r="U13" t="n">
         <v>0</v>
@@ -1325,47 +1349,49 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0</v>
+        <v>0.1940298467265662</v>
       </c>
       <c r="D14" t="n">
-        <v>0</v>
+        <v>2.899386359683304e-80</v>
       </c>
       <c r="E14" t="n">
-        <v>0.3217796385288239</v>
+        <v>0.6058722138404846</v>
       </c>
       <c r="F14" t="n">
-        <v>12.42500000000001</v>
+        <v>23.83684272300471</v>
       </c>
       <c r="G14" t="n">
-        <v>0.03944444444444444</v>
+        <v>0.3355555555555556</v>
       </c>
       <c r="H14" t="n">
-        <v>0</v>
+        <v>0.15</v>
       </c>
       <c r="I14" t="n">
-        <v>0</v>
-      </c>
-      <c r="J14" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J14" t="n">
+        <v>1</v>
+      </c>
       <c r="K14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L14" t="n">
         <v>0</v>
       </c>
       <c r="M14" t="n">
-        <v>0.05882352941176471</v>
+        <v>0.1549295774647887</v>
       </c>
       <c r="N14" t="n">
-        <v>0.002100467681884766</v>
+        <v>25.28776860237122</v>
       </c>
       <c r="O14" t="n">
-        <v>1122.66796875</v>
+        <v>1127.953125</v>
       </c>
       <c r="P14" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="Q14" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R14" t="n">
         <v>0</v>
@@ -1374,7 +1400,7 @@
         <v>0</v>
       </c>
       <c r="T14" t="n">
-        <v>0.002099275588989258</v>
+        <v>25.28776669502258</v>
       </c>
       <c r="U14" t="n">
         <v>0</v>
@@ -1390,47 +1416,49 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0</v>
+        <v>0.2169811270914917</v>
       </c>
       <c r="D15" t="n">
-        <v>0</v>
+        <v>0.03535154882114189</v>
       </c>
       <c r="E15" t="n">
-        <v>0.3361954092979431</v>
+        <v>0.5649368762969971</v>
       </c>
       <c r="F15" t="n">
-        <v>12.42500000000001</v>
+        <v>43.6460872528971</v>
       </c>
       <c r="G15" t="n">
-        <v>0.1428571428571428</v>
+        <v>1.223340040241449</v>
       </c>
       <c r="H15" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="I15" t="n">
-        <v>0</v>
-      </c>
-      <c r="J15" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J15" t="n">
+        <v>1</v>
+      </c>
       <c r="K15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L15" t="n">
         <v>0</v>
       </c>
       <c r="M15" t="n">
-        <v>0.06666666666666667</v>
+        <v>0.1509433962264151</v>
       </c>
       <c r="N15" t="n">
-        <v>0.002120256423950195</v>
+        <v>20.3046600818634</v>
       </c>
       <c r="O15" t="n">
-        <v>1122.66796875</v>
+        <v>1127.953125</v>
       </c>
       <c r="P15" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="Q15" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R15" t="n">
         <v>0</v>
@@ -1439,7 +1467,7 @@
         <v>0</v>
       </c>
       <c r="T15" t="n">
-        <v>0.002119064331054688</v>
+        <v>20.30465817451477</v>
       </c>
       <c r="U15" t="n">
         <v>0</v>
@@ -1455,27 +1483,29 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>0</v>
+        <v>0.2891566215125563</v>
       </c>
       <c r="D16" t="n">
-        <v>0</v>
+        <v>4.667647058635137e-155</v>
       </c>
       <c r="E16" t="n">
-        <v>0.3227388560771942</v>
+        <v>0.6510640382766724</v>
       </c>
       <c r="F16" t="n">
-        <v>12.42500000000001</v>
+        <v>47.20727272727277</v>
       </c>
       <c r="G16" t="n">
-        <v>0.101283880171184</v>
+        <v>1.002853067047076</v>
       </c>
       <c r="H16" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="I16" t="n">
-        <v>0</v>
-      </c>
-      <c r="J16" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J16" t="n">
+        <v>1</v>
+      </c>
       <c r="K16" t="n">
         <v>0</v>
       </c>
@@ -1483,19 +1513,19 @@
         <v>0</v>
       </c>
       <c r="M16" t="n">
-        <v>0.06666666666666667</v>
+        <v>0.25</v>
       </c>
       <c r="N16" t="n">
-        <v>0.001978874206542969</v>
+        <v>19.41476559638977</v>
       </c>
       <c r="O16" t="n">
-        <v>1122.66796875</v>
+        <v>1127.95703125</v>
       </c>
       <c r="P16" t="n">
-        <v>0</v>
+        <v>10.7</v>
       </c>
       <c r="Q16" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R16" t="n">
         <v>0</v>
@@ -1504,7 +1534,7 @@
         <v>0</v>
       </c>
       <c r="T16" t="n">
-        <v>0.001977920532226562</v>
+        <v>19.41476392745972</v>
       </c>
       <c r="U16" t="n">
         <v>0</v>
@@ -1520,47 +1550,49 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>0</v>
+        <v>0.158139530210925</v>
       </c>
       <c r="D17" t="n">
-        <v>0</v>
+        <v>3.534928643185659e-232</v>
       </c>
       <c r="E17" t="n">
-        <v>0.3224216401576996</v>
+        <v>0.5533502697944641</v>
       </c>
       <c r="F17" t="n">
-        <v>12.42500000000001</v>
+        <v>26.35875000000004</v>
       </c>
       <c r="G17" t="n">
-        <v>0.09543010752688172</v>
+        <v>0.6182795698924731</v>
       </c>
       <c r="H17" t="n">
-        <v>0</v>
+        <v>0.1428571428571428</v>
       </c>
       <c r="I17" t="n">
-        <v>0</v>
-      </c>
-      <c r="J17" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J17" t="n">
+        <v>1</v>
+      </c>
       <c r="K17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L17" t="n">
         <v>0</v>
       </c>
       <c r="M17" t="n">
-        <v>0.06666666666666667</v>
+        <v>0.1111111111111111</v>
       </c>
       <c r="N17" t="n">
-        <v>0.002335071563720703</v>
+        <v>21.44692516326904</v>
       </c>
       <c r="O17" t="n">
-        <v>1122.671875</v>
+        <v>1127.95703125</v>
       </c>
       <c r="P17" t="n">
-        <v>0</v>
+        <v>11.3</v>
       </c>
       <c r="Q17" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R17" t="n">
         <v>0</v>
@@ -1569,7 +1601,7 @@
         <v>0</v>
       </c>
       <c r="T17" t="n">
-        <v>0.002333641052246094</v>
+        <v>21.44692325592041</v>
       </c>
       <c r="U17" t="n">
         <v>0</v>
@@ -1585,47 +1617,49 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>0</v>
+        <v>0.2281368784272579</v>
       </c>
       <c r="D18" t="n">
-        <v>0</v>
+        <v>7.767617537256228e-80</v>
       </c>
       <c r="E18" t="n">
-        <v>0.3511787950992584</v>
+        <v>0.5974078774452209</v>
       </c>
       <c r="F18" t="n">
-        <v>12.42500000000001</v>
+        <v>37.71025412087914</v>
       </c>
       <c r="G18" t="n">
-        <v>0.02764797507788162</v>
+        <v>0.2858255451713396</v>
       </c>
       <c r="H18" t="n">
-        <v>0</v>
+        <v>0.625</v>
       </c>
       <c r="I18" t="n">
-        <v>0</v>
-      </c>
-      <c r="J18" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J18" t="n">
+        <v>1</v>
+      </c>
       <c r="K18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L18" t="n">
         <v>0</v>
       </c>
       <c r="M18" t="n">
-        <v>0.09090909090909091</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="N18" t="n">
-        <v>0.001950502395629883</v>
+        <v>23.94958305358887</v>
       </c>
       <c r="O18" t="n">
-        <v>1122.6796875</v>
+        <v>1127.95703125</v>
       </c>
       <c r="P18" t="n">
-        <v>25</v>
+        <v>11.4</v>
       </c>
       <c r="Q18" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R18" t="n">
         <v>0</v>
@@ -1634,7 +1668,7 @@
         <v>0</v>
       </c>
       <c r="T18" t="n">
-        <v>0.001949548721313477</v>
+        <v>23.94958162307739</v>
       </c>
       <c r="U18" t="n">
         <v>0</v>
@@ -1650,47 +1684,49 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>0</v>
+        <v>0.1976047865099143</v>
       </c>
       <c r="D19" t="n">
-        <v>0</v>
+        <v>2.887729973462374e-80</v>
       </c>
       <c r="E19" t="n">
-        <v>0.3164240121841431</v>
+        <v>0.601162850856781</v>
       </c>
       <c r="F19" t="n">
-        <v>12.42500000000001</v>
+        <v>27.60816425120777</v>
       </c>
       <c r="G19" t="n">
-        <v>0.04680290046143705</v>
+        <v>0.3328938694792353</v>
       </c>
       <c r="H19" t="n">
         <v>0</v>
       </c>
       <c r="I19" t="n">
-        <v>0</v>
-      </c>
-      <c r="J19" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J19" t="n">
+        <v>1</v>
+      </c>
       <c r="K19" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="L19" t="n">
         <v>0</v>
       </c>
       <c r="M19" t="n">
-        <v>0.05882352941176471</v>
+        <v>0.2125984251968504</v>
       </c>
       <c r="N19" t="n">
-        <v>0.002282619476318359</v>
+        <v>23.09705519676208</v>
       </c>
       <c r="O19" t="n">
-        <v>1122.703125</v>
+        <v>1127.95703125</v>
       </c>
       <c r="P19" t="n">
-        <v>0</v>
+        <v>10.7</v>
       </c>
       <c r="Q19" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R19" t="n">
         <v>0</v>
@@ -1699,7 +1735,7 @@
         <v>0</v>
       </c>
       <c r="T19" t="n">
-        <v>0.002281427383422852</v>
+        <v>23.09705352783203</v>
       </c>
       <c r="U19" t="n">
         <v>0</v>
@@ -1715,47 +1751,49 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>0.008032128120514206</v>
+        <v>0.2125340554890155</v>
       </c>
       <c r="D20" t="n">
-        <v>1.21304235279905e-268</v>
+        <v>0.01244871695417394</v>
       </c>
       <c r="E20" t="n">
-        <v>0.3357276916503906</v>
+        <v>0.5857091546058655</v>
       </c>
       <c r="F20" t="n">
-        <v>12.42500000000001</v>
+        <v>28.75781835205996</v>
       </c>
       <c r="G20" t="n">
-        <v>0.05039034776437189</v>
+        <v>0.4996451383960255</v>
       </c>
       <c r="H20" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="I20" t="n">
-        <v>0</v>
-      </c>
-      <c r="J20" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J20" t="n">
+        <v>1</v>
+      </c>
       <c r="K20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L20" t="n">
         <v>0</v>
       </c>
       <c r="M20" t="n">
-        <v>0.05263157894736842</v>
+        <v>0.1603053435114504</v>
       </c>
       <c r="N20" t="n">
-        <v>0.002015590667724609</v>
+        <v>22.91807460784912</v>
       </c>
       <c r="O20" t="n">
-        <v>1122.70703125</v>
+        <v>1127.98046875</v>
       </c>
       <c r="P20" t="n">
-        <v>0</v>
+        <v>10.8</v>
       </c>
       <c r="Q20" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R20" t="n">
         <v>0</v>
@@ -1764,7 +1802,7 @@
         <v>0</v>
       </c>
       <c r="T20" t="n">
-        <v>0.002014636993408203</v>
+        <v>22.91807198524475</v>
       </c>
       <c r="U20" t="n">
         <v>0</v>
@@ -1780,47 +1818,49 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>0</v>
+        <v>0.1588235257515572</v>
       </c>
       <c r="D21" t="n">
-        <v>0</v>
+        <v>4.668372612564776e-157</v>
       </c>
       <c r="E21" t="n">
-        <v>0.3344107270240784</v>
+        <v>0.5306360721588135</v>
       </c>
       <c r="F21" t="n">
-        <v>12.42500000000001</v>
+        <v>22.23763506625895</v>
       </c>
       <c r="G21" t="n">
-        <v>0.04022662889518414</v>
+        <v>0.2770538243626062</v>
       </c>
       <c r="H21" t="n">
         <v>0</v>
       </c>
       <c r="I21" t="n">
-        <v>0</v>
-      </c>
-      <c r="J21" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J21" t="n">
+        <v>0.125</v>
+      </c>
       <c r="K21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L21" t="n">
         <v>0</v>
       </c>
       <c r="M21" t="n">
-        <v>0.0136986301369863</v>
+        <v>0.03940886699507389</v>
       </c>
       <c r="N21" t="n">
-        <v>0.003462791442871094</v>
+        <v>39.67655372619629</v>
       </c>
       <c r="O21" t="n">
-        <v>1122.84765625</v>
+        <v>1128.32421875</v>
       </c>
       <c r="P21" t="n">
-        <v>0</v>
+        <v>11.2</v>
       </c>
       <c r="Q21" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R21" t="n">
         <v>0</v>
@@ -1829,7 +1869,7 @@
         <v>0</v>
       </c>
       <c r="T21" t="n">
-        <v>0.003460884094238281</v>
+        <v>39.67655181884766</v>
       </c>
       <c r="U21" t="n">
         <v>0</v>
@@ -1845,47 +1885,49 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>0</v>
+        <v>0.3294663524765694</v>
       </c>
       <c r="D22" t="n">
-        <v>0</v>
+        <v>7.278906466481833e-79</v>
       </c>
       <c r="E22" t="n">
-        <v>0.3496818244457245</v>
+        <v>0.6370041370391846</v>
       </c>
       <c r="F22" t="n">
-        <v>12.42500000000001</v>
+        <v>34.80610502418324</v>
       </c>
       <c r="G22" t="n">
-        <v>0.04303030303030303</v>
+        <v>0.6387878787878788</v>
       </c>
       <c r="H22" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="I22" t="n">
-        <v>0</v>
-      </c>
-      <c r="J22" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J22" t="n">
+        <v>1</v>
+      </c>
       <c r="K22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L22" t="n">
         <v>0</v>
       </c>
       <c r="M22" t="n">
-        <v>0.05263157894736842</v>
+        <v>0.2647058823529412</v>
       </c>
       <c r="N22" t="n">
-        <v>0.002453804016113281</v>
+        <v>32.27557349205017</v>
       </c>
       <c r="O22" t="n">
-        <v>1122.8515625</v>
+        <v>1128.32421875</v>
       </c>
       <c r="P22" t="n">
-        <v>0</v>
+        <v>11.8</v>
       </c>
       <c r="Q22" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R22" t="n">
         <v>0</v>
@@ -1894,7 +1936,7 @@
         <v>0</v>
       </c>
       <c r="T22" t="n">
-        <v>0.002452373504638672</v>
+        <v>32.27557182312012</v>
       </c>
       <c r="U22" t="n">
         <v>0</v>
@@ -1910,47 +1952,49 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>0.005847952928251443</v>
+        <v>0.1716937320882209</v>
       </c>
       <c r="D23" t="n">
-        <v>1.811128572821972e-307</v>
+        <v>0.0002153634457716161</v>
       </c>
       <c r="E23" t="n">
-        <v>0.3417599201202393</v>
+        <v>0.5935307741165161</v>
       </c>
       <c r="F23" t="n">
-        <v>12.42500000000001</v>
+        <v>34.42153434800497</v>
       </c>
       <c r="G23" t="n">
-        <v>0.03261368856224162</v>
+        <v>0.2668810289389068</v>
       </c>
       <c r="H23" t="n">
-        <v>0</v>
+        <v>0.07142857142857142</v>
       </c>
       <c r="I23" t="n">
-        <v>0</v>
-      </c>
-      <c r="J23" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J23" t="n">
+        <v>1</v>
+      </c>
       <c r="K23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L23" t="n">
         <v>0</v>
       </c>
       <c r="M23" t="n">
-        <v>0.09090909090909091</v>
+        <v>0.2708333333333334</v>
       </c>
       <c r="N23" t="n">
-        <v>0.002390623092651367</v>
+        <v>32.10565423965454</v>
       </c>
       <c r="O23" t="n">
-        <v>1122.85546875</v>
+        <v>1128.32421875</v>
       </c>
       <c r="P23" t="n">
-        <v>25</v>
+        <v>10.6</v>
       </c>
       <c r="Q23" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R23" t="n">
         <v>0</v>
@@ -1959,7 +2003,7 @@
         <v>0</v>
       </c>
       <c r="T23" t="n">
-        <v>0.002389192581176758</v>
+        <v>32.10565137863159</v>
       </c>
       <c r="U23" t="n">
         <v>0</v>
@@ -1975,47 +2019,49 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>0</v>
+        <v>0.2333333284222223</v>
       </c>
       <c r="D24" t="n">
-        <v>0</v>
+        <v>0.02289964820840968</v>
       </c>
       <c r="E24" t="n">
-        <v>0.3145212233066559</v>
+        <v>0.6228812336921692</v>
       </c>
       <c r="F24" t="n">
-        <v>12.42500000000001</v>
+        <v>40.53012682137077</v>
       </c>
       <c r="G24" t="n">
-        <v>0.109062980030722</v>
+        <v>1.288786482334869</v>
       </c>
       <c r="H24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I24" t="n">
-        <v>0</v>
-      </c>
-      <c r="J24" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J24" t="n">
+        <v>1</v>
+      </c>
       <c r="K24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L24" t="n">
         <v>0</v>
       </c>
       <c r="M24" t="n">
-        <v>0.07692307692307693</v>
+        <v>0.3388429752066116</v>
       </c>
       <c r="N24" t="n">
-        <v>0.001929044723510742</v>
+        <v>19.40041732788086</v>
       </c>
       <c r="O24" t="n">
-        <v>1122.85546875</v>
+        <v>1128.32421875</v>
       </c>
       <c r="P24" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="Q24" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R24" t="n">
         <v>0</v>
@@ -2024,7 +2070,7 @@
         <v>0</v>
       </c>
       <c r="T24" t="n">
-        <v>0.001927614212036133</v>
+        <v>19.40041542053223</v>
       </c>
       <c r="U24" t="n">
         <v>0</v>
@@ -2040,47 +2086,49 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>0</v>
+        <v>0.2977099187585223</v>
       </c>
       <c r="D25" t="n">
-        <v>0</v>
+        <v>1.030439770766457e-78</v>
       </c>
       <c r="E25" t="n">
-        <v>0.3218568563461304</v>
+        <v>0.6429927349090576</v>
       </c>
       <c r="F25" t="n">
-        <v>12.42500000000001</v>
+        <v>47.54985829959514</v>
       </c>
       <c r="G25" t="n">
-        <v>0.1070889894419306</v>
+        <v>1.253393665158371</v>
       </c>
       <c r="H25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I25" t="n">
-        <v>0</v>
-      </c>
-      <c r="J25" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J25" t="n">
+        <v>1</v>
+      </c>
       <c r="K25" t="n">
-        <v>0</v>
+        <v>0.75</v>
       </c>
       <c r="L25" t="n">
         <v>0</v>
       </c>
       <c r="M25" t="n">
-        <v>0.1111111111111111</v>
+        <v>0.3670886075949367</v>
       </c>
       <c r="N25" t="n">
-        <v>0.002121925354003906</v>
+        <v>18.13336539268494</v>
       </c>
       <c r="O25" t="n">
-        <v>1122.85546875</v>
+        <v>1128.32421875</v>
       </c>
       <c r="P25" t="n">
-        <v>0</v>
+        <v>10.8</v>
       </c>
       <c r="Q25" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R25" t="n">
         <v>0</v>
@@ -2089,7 +2137,7 @@
         <v>0</v>
       </c>
       <c r="T25" t="n">
-        <v>0.002120494842529297</v>
+        <v>18.13336372375488</v>
       </c>
       <c r="U25" t="n">
         <v>0</v>
@@ -2105,47 +2153,49 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>0</v>
+        <v>0.2660550409540444</v>
       </c>
       <c r="D26" t="n">
-        <v>0</v>
+        <v>1.178485891180151e-78</v>
       </c>
       <c r="E26" t="n">
-        <v>0.3182421326637268</v>
+        <v>0.6297150850296021</v>
       </c>
       <c r="F26" t="n">
-        <v>12.42500000000001</v>
+        <v>40.08553278688524</v>
       </c>
       <c r="G26" t="n">
-        <v>0.123050259965338</v>
+        <v>1.162911611785095</v>
       </c>
       <c r="H26" t="n">
         <v>0</v>
       </c>
       <c r="I26" t="n">
-        <v>0</v>
-      </c>
-      <c r="J26" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J26" t="n">
+        <v>1</v>
+      </c>
       <c r="K26" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L26" t="n">
         <v>0</v>
       </c>
       <c r="M26" t="n">
-        <v>0.1111111111111111</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="N26" t="n">
-        <v>0.001860857009887695</v>
+        <v>19.86343383789062</v>
       </c>
       <c r="O26" t="n">
-        <v>1122.85546875</v>
+        <v>1128.32421875</v>
       </c>
       <c r="P26" t="n">
-        <v>25</v>
+        <v>11.5</v>
       </c>
       <c r="Q26" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R26" t="n">
         <v>0</v>
@@ -2154,7 +2204,7 @@
         <v>0</v>
       </c>
       <c r="T26" t="n">
-        <v>0.001859664916992188</v>
+        <v>19.86343216896057</v>
       </c>
       <c r="U26" t="n">
         <v>0</v>
@@ -2170,47 +2220,49 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>0</v>
+        <v>0.3605150164998436</v>
       </c>
       <c r="D27" t="n">
-        <v>0</v>
+        <v>0.1186020801410399</v>
       </c>
       <c r="E27" t="n">
-        <v>0.3122285008430481</v>
+        <v>0.6553923487663269</v>
       </c>
       <c r="F27" t="n">
-        <v>12.42500000000001</v>
+        <v>35.95960304054054</v>
       </c>
       <c r="G27" t="n">
-        <v>0.09712722298221614</v>
+        <v>0.905608755129959</v>
       </c>
       <c r="H27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I27" t="n">
-        <v>0</v>
-      </c>
-      <c r="J27" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J27" t="n">
+        <v>1</v>
+      </c>
       <c r="K27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L27" t="n">
         <v>0</v>
       </c>
       <c r="M27" t="n">
-        <v>0.1111111111111111</v>
+        <v>0.4252873563218391</v>
       </c>
       <c r="N27" t="n">
-        <v>0.002106189727783203</v>
+        <v>18.10218620300293</v>
       </c>
       <c r="O27" t="n">
-        <v>1122.85546875</v>
+        <v>1128.32421875</v>
       </c>
       <c r="P27" t="n">
-        <v>0</v>
+        <v>10.8</v>
       </c>
       <c r="Q27" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R27" t="n">
         <v>0</v>
@@ -2219,7 +2271,7 @@
         <v>0</v>
       </c>
       <c r="T27" t="n">
-        <v>0.002104759216308594</v>
+        <v>18.10218143463135</v>
       </c>
       <c r="U27" t="n">
         <v>0</v>
@@ -2235,47 +2287,49 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>0</v>
+        <v>0.2361623567614821</v>
       </c>
       <c r="D28" t="n">
-        <v>0</v>
+        <v>4.645779704255236e-155</v>
       </c>
       <c r="E28" t="n">
-        <v>0.3209810554981232</v>
+        <v>0.6078421473503113</v>
       </c>
       <c r="F28" t="n">
-        <v>12.42500000000001</v>
+        <v>27.47001287415517</v>
       </c>
       <c r="G28" t="n">
-        <v>0.1075757575757576</v>
+        <v>1.31969696969697</v>
       </c>
       <c r="H28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I28" t="n">
-        <v>0</v>
-      </c>
-      <c r="J28" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J28" t="n">
+        <v>1</v>
+      </c>
       <c r="K28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L28" t="n">
         <v>0</v>
       </c>
       <c r="M28" t="n">
-        <v>0.1111111111111111</v>
+        <v>0.3749999999999999</v>
       </c>
       <c r="N28" t="n">
-        <v>0.001869440078735352</v>
+        <v>18.35174608230591</v>
       </c>
       <c r="O28" t="n">
-        <v>1122.85546875</v>
+        <v>1128.32421875</v>
       </c>
       <c r="P28" t="n">
-        <v>0</v>
+        <v>12.3</v>
       </c>
       <c r="Q28" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R28" t="n">
         <v>0</v>
@@ -2284,7 +2338,7 @@
         <v>0</v>
       </c>
       <c r="T28" t="n">
-        <v>0.001868009567260742</v>
+        <v>18.3517439365387</v>
       </c>
       <c r="U28" t="n">
         <v>0</v>
@@ -2300,47 +2354,49 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>0</v>
+        <v>0.265402838651423</v>
       </c>
       <c r="D29" t="n">
-        <v>0</v>
+        <v>3.729438571895397e-155</v>
       </c>
       <c r="E29" t="n">
-        <v>0.317456990480423</v>
+        <v>0.6346973776817322</v>
       </c>
       <c r="F29" t="n">
-        <v>12.42500000000001</v>
+        <v>38.85805031446543</v>
       </c>
       <c r="G29" t="n">
-        <v>0.1232638888888889</v>
+        <v>1.071180555555556</v>
       </c>
       <c r="H29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I29" t="n">
-        <v>0</v>
-      </c>
-      <c r="J29" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J29" t="n">
+        <v>1</v>
+      </c>
       <c r="K29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L29" t="n">
         <v>0</v>
       </c>
       <c r="M29" t="n">
-        <v>0.1111111111111111</v>
+        <v>0.2</v>
       </c>
       <c r="N29" t="n">
-        <v>0.002075672149658203</v>
+        <v>19.92830324172974</v>
       </c>
       <c r="O29" t="n">
-        <v>1122.859375</v>
+        <v>1128.32421875</v>
       </c>
       <c r="P29" t="n">
-        <v>0</v>
+        <v>10.2</v>
       </c>
       <c r="Q29" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R29" t="n">
         <v>0</v>
@@ -2349,7 +2405,7 @@
         <v>0</v>
       </c>
       <c r="T29" t="n">
-        <v>0.002074480056762695</v>
+        <v>19.92830109596252</v>
       </c>
       <c r="U29" t="n">
         <v>0</v>
@@ -2365,47 +2421,49 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>0</v>
+        <v>0.04733727709814085</v>
       </c>
       <c r="D30" t="n">
-        <v>0</v>
+        <v>1.349112716410584e-155</v>
       </c>
       <c r="E30" t="n">
-        <v>0.4068427383899689</v>
+        <v>0.416518896818161</v>
       </c>
       <c r="F30" t="n">
-        <v>12.42500000000001</v>
+        <v>36.02919354838713</v>
       </c>
       <c r="G30" t="n">
-        <v>0.71</v>
+        <v>9.130000000000001</v>
       </c>
       <c r="H30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I30" t="n">
-        <v>0</v>
-      </c>
-      <c r="J30" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J30" t="n">
+        <v>1</v>
+      </c>
       <c r="K30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L30" t="n">
         <v>0</v>
       </c>
       <c r="M30" t="n">
-        <v>0.06666666666666667</v>
+        <v>0.25</v>
       </c>
       <c r="N30" t="n">
-        <v>0.002249240875244141</v>
+        <v>19.22996735572815</v>
       </c>
       <c r="O30" t="n">
-        <v>1122.859375</v>
+        <v>1128.32421875</v>
       </c>
       <c r="P30" t="n">
-        <v>0</v>
+        <v>12.1</v>
       </c>
       <c r="Q30" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R30" t="n">
         <v>0</v>
@@ -2414,7 +2472,7 @@
         <v>0</v>
       </c>
       <c r="T30" t="n">
-        <v>0.002248048782348633</v>
+        <v>19.22996592521667</v>
       </c>
       <c r="U30" t="n">
         <v>0</v>
@@ -2430,47 +2488,49 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>0</v>
+        <v>0.06289308069301057</v>
       </c>
       <c r="D31" t="n">
-        <v>0</v>
+        <v>1.482112406539712e-155</v>
       </c>
       <c r="E31" t="n">
-        <v>0.405496746301651</v>
+        <v>0.4403652250766754</v>
       </c>
       <c r="F31" t="n">
-        <v>12.42500000000001</v>
+        <v>34.22715789473688</v>
       </c>
       <c r="G31" t="n">
-        <v>0.6893203883495146</v>
+        <v>8.25242718446602</v>
       </c>
       <c r="H31" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="I31" t="n">
-        <v>0</v>
-      </c>
-      <c r="J31" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J31" t="n">
+        <v>1</v>
+      </c>
       <c r="K31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L31" t="n">
         <v>0</v>
       </c>
       <c r="M31" t="n">
-        <v>0.06666666666666667</v>
+        <v>0.2436974789915966</v>
       </c>
       <c r="N31" t="n">
-        <v>0.001905918121337891</v>
+        <v>18.89662933349609</v>
       </c>
       <c r="O31" t="n">
-        <v>1122.859375</v>
+        <v>1128.32421875</v>
       </c>
       <c r="P31" t="n">
-        <v>33.3</v>
+        <v>10.7</v>
       </c>
       <c r="Q31" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R31" t="n">
         <v>0</v>
@@ -2479,7 +2539,7 @@
         <v>0</v>
       </c>
       <c r="T31" t="n">
-        <v>0.001904964447021484</v>
+        <v>18.89662766456604</v>
       </c>
       <c r="U31" t="n">
         <v>0</v>
@@ -2495,47 +2555,49 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>0</v>
+        <v>0.098039214077278</v>
       </c>
       <c r="D32" t="n">
-        <v>0</v>
+        <v>1.960114543996295e-155</v>
       </c>
       <c r="E32" t="n">
-        <v>0.4001372754573822</v>
+        <v>0.4697017669677734</v>
       </c>
       <c r="F32" t="n">
-        <v>12.42500000000001</v>
+        <v>38.82620155038765</v>
       </c>
       <c r="G32" t="n">
-        <v>0.71</v>
+        <v>5.5</v>
       </c>
       <c r="H32" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I32" t="n">
-        <v>0</v>
-      </c>
-      <c r="J32" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J32" t="n">
+        <v>1</v>
+      </c>
       <c r="K32" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L32" t="n">
         <v>0</v>
       </c>
       <c r="M32" t="n">
-        <v>0.06666666666666667</v>
+        <v>0.2</v>
       </c>
       <c r="N32" t="n">
-        <v>0.002118587493896484</v>
+        <v>19.64923572540283</v>
       </c>
       <c r="O32" t="n">
-        <v>1122.859375</v>
+        <v>1128.32421875</v>
       </c>
       <c r="P32" t="n">
-        <v>0</v>
+        <v>11.6</v>
       </c>
       <c r="Q32" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R32" t="n">
         <v>0</v>
@@ -2544,7 +2606,7 @@
         <v>0</v>
       </c>
       <c r="T32" t="n">
-        <v>0.002117395401000977</v>
+        <v>19.64923357963562</v>
       </c>
       <c r="U32" t="n">
         <v>0</v>
@@ -2560,19 +2622,19 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>0</v>
+        <v>0.1626016211117723</v>
       </c>
       <c r="D33" t="n">
-        <v>0</v>
+        <v>2.643833696368049e-155</v>
       </c>
       <c r="E33" t="n">
-        <v>0.3932636678218842</v>
+        <v>0.5117695927619934</v>
       </c>
       <c r="F33" t="n">
-        <v>12.42500000000001</v>
+        <v>35.00630612244899</v>
       </c>
       <c r="G33" t="n">
-        <v>0.1966759002770083</v>
+        <v>1.157894736842105</v>
       </c>
       <c r="H33" t="n">
         <v>0</v>
@@ -2580,27 +2642,29 @@
       <c r="I33" t="n">
         <v>0</v>
       </c>
-      <c r="J33" t="inlineStr"/>
+      <c r="J33" t="n">
+        <v>0</v>
+      </c>
       <c r="K33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L33" t="n">
         <v>0</v>
       </c>
       <c r="M33" t="n">
-        <v>0.07692307692307693</v>
+        <v>0.1578947368421053</v>
       </c>
       <c r="N33" t="n">
-        <v>0.002054452896118164</v>
+        <v>22.60587668418884</v>
       </c>
       <c r="O33" t="n">
-        <v>1122.859375</v>
+        <v>1128.32421875</v>
       </c>
       <c r="P33" t="n">
-        <v>0</v>
+        <v>11.3</v>
       </c>
       <c r="Q33" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R33" t="n">
         <v>0</v>
@@ -2609,7 +2673,7 @@
         <v>0</v>
       </c>
       <c r="T33" t="n">
-        <v>0.002053260803222656</v>
+        <v>22.60587501525879</v>
       </c>
       <c r="U33" t="n">
         <v>0</v>
@@ -2625,47 +2689,49 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>0</v>
+        <v>0.2285714236480727</v>
       </c>
       <c r="D34" t="n">
-        <v>0</v>
+        <v>2.005256986190514e-155</v>
       </c>
       <c r="E34" t="n">
-        <v>0.3809874057769775</v>
+        <v>0.5366058349609375</v>
       </c>
       <c r="F34" t="n">
-        <v>12.42500000000001</v>
+        <v>30.21060344827589</v>
       </c>
       <c r="G34" t="n">
-        <v>0.1031976744186047</v>
+        <v>0.7252906976744186</v>
       </c>
       <c r="H34" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="I34" t="n">
-        <v>0</v>
-      </c>
-      <c r="J34" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J34" t="n">
+        <v>1</v>
+      </c>
       <c r="K34" t="n">
-        <v>0</v>
+        <v>0.75</v>
       </c>
       <c r="L34" t="n">
         <v>0</v>
       </c>
       <c r="M34" t="n">
-        <v>0.1111111111111111</v>
+        <v>0.1549295774647887</v>
       </c>
       <c r="N34" t="n">
-        <v>0.002185583114624023</v>
+        <v>22.19046759605408</v>
       </c>
       <c r="O34" t="n">
-        <v>1122.859375</v>
+        <v>1128.32421875</v>
       </c>
       <c r="P34" t="n">
-        <v>25</v>
+        <v>10.8</v>
       </c>
       <c r="Q34" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R34" t="n">
         <v>0</v>
@@ -2674,7 +2740,7 @@
         <v>0</v>
       </c>
       <c r="T34" t="n">
-        <v>0.002184629440307617</v>
+        <v>22.1904661655426</v>
       </c>
       <c r="U34" t="n">
         <v>0</v>
@@ -2690,47 +2756,49 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>0</v>
+        <v>0.2307692261491207</v>
       </c>
       <c r="D35" t="n">
-        <v>0</v>
+        <v>1.456281036629997e-155</v>
       </c>
       <c r="E35" t="n">
-        <v>0.3331394195556641</v>
+        <v>0.5998542308807373</v>
       </c>
       <c r="F35" t="n">
-        <v>12.42500000000001</v>
+        <v>23.42578859060401</v>
       </c>
       <c r="G35" t="n">
-        <v>0.06217162872154115</v>
+        <v>0.5621716287215411</v>
       </c>
       <c r="H35" t="n">
-        <v>0</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="I35" t="n">
-        <v>0</v>
-      </c>
-      <c r="J35" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J35" t="n">
+        <v>1</v>
+      </c>
       <c r="K35" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L35" t="n">
         <v>0</v>
       </c>
       <c r="M35" t="n">
-        <v>0.06666666666666667</v>
+        <v>0.1891891891891892</v>
       </c>
       <c r="N35" t="n">
-        <v>0.001955747604370117</v>
+        <v>19.71259593963623</v>
       </c>
       <c r="O35" t="n">
-        <v>1122.859375</v>
+        <v>1128.32421875</v>
       </c>
       <c r="P35" t="n">
-        <v>25</v>
+        <v>11.5</v>
       </c>
       <c r="Q35" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R35" t="n">
         <v>0</v>
@@ -2739,7 +2807,7 @@
         <v>0</v>
       </c>
       <c r="T35" t="n">
-        <v>0.001954793930053711</v>
+        <v>19.71259379386902</v>
       </c>
       <c r="U35" t="n">
         <v>0</v>
@@ -2755,47 +2823,49 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>0</v>
+        <v>0.2153846104204143</v>
       </c>
       <c r="D36" t="n">
-        <v>0</v>
+        <v>2.459398402756693e-155</v>
       </c>
       <c r="E36" t="n">
-        <v>0.3015691339969635</v>
+        <v>0.5755105018615723</v>
       </c>
       <c r="F36" t="n">
-        <v>12.42500000000001</v>
+        <v>17.82568102073367</v>
       </c>
       <c r="G36" t="n">
-        <v>0.1125198098256735</v>
+        <v>1.245641838351822</v>
       </c>
       <c r="H36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I36" t="n">
-        <v>0</v>
-      </c>
-      <c r="J36" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J36" t="n">
+        <v>1</v>
+      </c>
       <c r="K36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L36" t="n">
         <v>0</v>
       </c>
       <c r="M36" t="n">
-        <v>0.06666666666666667</v>
+        <v>0.1891891891891892</v>
       </c>
       <c r="N36" t="n">
-        <v>0.002138137817382812</v>
+        <v>19.07508730888367</v>
       </c>
       <c r="O36" t="n">
-        <v>1122.859375</v>
+        <v>1128.32421875</v>
       </c>
       <c r="P36" t="n">
-        <v>0</v>
+        <v>10.7</v>
       </c>
       <c r="Q36" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R36" t="n">
         <v>0</v>
@@ -2804,7 +2874,7 @@
         <v>0</v>
       </c>
       <c r="T36" t="n">
-        <v>0.002137184143066406</v>
+        <v>19.07508492469788</v>
       </c>
       <c r="U36" t="n">
         <v>0</v>
@@ -2820,47 +2890,49 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>0</v>
+        <v>0.2452830138697046</v>
       </c>
       <c r="D37" t="n">
-        <v>0</v>
+        <v>1.359833238477108e-78</v>
       </c>
       <c r="E37" t="n">
-        <v>0.3549112677574158</v>
+        <v>0.6297886371612549</v>
       </c>
       <c r="F37" t="n">
-        <v>12.42500000000001</v>
+        <v>37.90426900584799</v>
       </c>
       <c r="G37" t="n">
-        <v>0.07529162248144221</v>
+        <v>1.091198303287381</v>
       </c>
       <c r="H37" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I37" t="n">
-        <v>0</v>
-      </c>
-      <c r="J37" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J37" t="n">
+        <v>1</v>
+      </c>
       <c r="K37" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L37" t="n">
         <v>0</v>
       </c>
       <c r="M37" t="n">
-        <v>0.1111111111111111</v>
+        <v>0.4845360824742268</v>
       </c>
       <c r="N37" t="n">
-        <v>0.00200963020324707</v>
+        <v>26.74604058265686</v>
       </c>
       <c r="O37" t="n">
-        <v>1122.859375</v>
+        <v>1128.32421875</v>
       </c>
       <c r="P37" t="n">
-        <v>0</v>
+        <v>11.3</v>
       </c>
       <c r="Q37" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R37" t="n">
         <v>0</v>
@@ -2869,7 +2941,7 @@
         <v>0</v>
       </c>
       <c r="T37" t="n">
-        <v>0.002008676528930664</v>
+        <v>26.74603891372681</v>
       </c>
       <c r="U37" t="n">
         <v>0</v>
@@ -2885,47 +2957,49 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>0</v>
+        <v>0.2159999950028801</v>
       </c>
       <c r="D38" t="n">
-        <v>0</v>
+        <v>4.177942492722784e-155</v>
       </c>
       <c r="E38" t="n">
-        <v>0.353282243013382</v>
+        <v>0.5601202249526978</v>
       </c>
       <c r="F38" t="n">
-        <v>12.42500000000001</v>
+        <v>14.27382022471912</v>
       </c>
       <c r="G38" t="n">
-        <v>0.09184993531694696</v>
+        <v>0.944372574385511</v>
       </c>
       <c r="H38" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="I38" t="n">
-        <v>0</v>
-      </c>
-      <c r="J38" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J38" t="n">
+        <v>1</v>
+      </c>
       <c r="K38" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L38" t="n">
         <v>0</v>
       </c>
       <c r="M38" t="n">
-        <v>0.09090909090909091</v>
+        <v>0.2708333333333334</v>
       </c>
       <c r="N38" t="n">
-        <v>0.002190589904785156</v>
+        <v>22.3070924282074</v>
       </c>
       <c r="O38" t="n">
-        <v>1122.859375</v>
+        <v>1128.32421875</v>
       </c>
       <c r="P38" t="n">
-        <v>0</v>
+        <v>11.4</v>
       </c>
       <c r="Q38" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R38" t="n">
         <v>0</v>
@@ -2934,7 +3008,7 @@
         <v>0</v>
       </c>
       <c r="T38" t="n">
-        <v>0.00218963623046875</v>
+        <v>22.30709004402161</v>
       </c>
       <c r="U38" t="n">
         <v>0</v>
@@ -2950,47 +3024,49 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>0</v>
+        <v>0.1729729681519359</v>
       </c>
       <c r="D39" t="n">
-        <v>0</v>
+        <v>2.690253750949746e-155</v>
       </c>
       <c r="E39" t="n">
-        <v>0.3316194117069244</v>
+        <v>0.5925518274307251</v>
       </c>
       <c r="F39" t="n">
-        <v>12.42500000000001</v>
+        <v>41.14184210526318</v>
       </c>
       <c r="G39" t="n">
-        <v>0.1047197640117994</v>
+        <v>0.6887905604719764</v>
       </c>
       <c r="H39" t="n">
-        <v>0</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="I39" t="n">
-        <v>0</v>
-      </c>
-      <c r="J39" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J39" t="n">
+        <v>0</v>
+      </c>
       <c r="K39" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L39" t="n">
         <v>0</v>
       </c>
       <c r="M39" t="n">
-        <v>0.05263157894736842</v>
+        <v>0.1452991452991453</v>
       </c>
       <c r="N39" t="n">
-        <v>0.05113697052001953</v>
+        <v>19.89927005767822</v>
       </c>
       <c r="O39" t="n">
-        <v>1122.859375</v>
+        <v>1128.32421875</v>
       </c>
       <c r="P39" t="n">
-        <v>0</v>
+        <v>12.1</v>
       </c>
       <c r="Q39" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R39" t="n">
         <v>0</v>
@@ -2999,7 +3075,7 @@
         <v>0</v>
       </c>
       <c r="T39" t="n">
-        <v>0.0511329174041748</v>
+        <v>19.89926767349243</v>
       </c>
       <c r="U39" t="n">
         <v>0</v>
@@ -3015,47 +3091,49 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>0</v>
+        <v>0.2262773673397625</v>
       </c>
       <c r="D40" t="n">
-        <v>0</v>
+        <v>3.711174997260935e-79</v>
       </c>
       <c r="E40" t="n">
-        <v>0.2845998406410217</v>
+        <v>0.523645281791687</v>
       </c>
       <c r="F40" t="n">
-        <v>12.42500000000001</v>
+        <v>25.17939393939398</v>
       </c>
       <c r="G40" t="n">
-        <v>0.07819383259911894</v>
+        <v>0.7026431718061674</v>
       </c>
       <c r="H40" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I40" t="n">
         <v>1</v>
       </c>
-      <c r="J40" t="inlineStr"/>
+      <c r="J40" t="n">
+        <v>1</v>
+      </c>
       <c r="K40" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="L40" t="n">
         <v>0</v>
       </c>
       <c r="M40" t="n">
-        <v>0.1111111111111111</v>
+        <v>0.2307692307692308</v>
       </c>
       <c r="N40" t="n">
-        <v>0.002626180648803711</v>
+        <v>19.04356861114502</v>
       </c>
       <c r="O40" t="n">
-        <v>1122.859375</v>
+        <v>1128.32421875</v>
       </c>
       <c r="P40" t="n">
-        <v>25</v>
+        <v>10.8</v>
       </c>
       <c r="Q40" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R40" t="n">
         <v>0</v>
@@ -3064,7 +3142,7 @@
         <v>0</v>
       </c>
       <c r="T40" t="n">
-        <v>0.002624750137329102</v>
+        <v>19.04356694221497</v>
       </c>
       <c r="U40" t="n">
         <v>0</v>
@@ -3080,47 +3158,49 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>0</v>
+        <v>0.1989528751251337</v>
       </c>
       <c r="D41" t="n">
-        <v>0</v>
+        <v>1.511314035121895e-79</v>
       </c>
       <c r="E41" t="n">
-        <v>0.2805698215961456</v>
+        <v>0.5371474027633667</v>
       </c>
       <c r="F41" t="n">
-        <v>12.42500000000001</v>
+        <v>31.28214245810057</v>
       </c>
       <c r="G41" t="n">
-        <v>0.04869684499314129</v>
+        <v>0.4917695473251029</v>
       </c>
       <c r="H41" t="n">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="I41" t="n">
         <v>1</v>
       </c>
-      <c r="J41" t="inlineStr"/>
+      <c r="J41" t="n">
+        <v>1</v>
+      </c>
       <c r="K41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L41" t="n">
         <v>0</v>
       </c>
       <c r="M41" t="n">
-        <v>0.1111111111111111</v>
+        <v>0.2405063291139241</v>
       </c>
       <c r="N41" t="n">
-        <v>0.00193476676940918</v>
+        <v>22.51703143119812</v>
       </c>
       <c r="O41" t="n">
-        <v>1122.859375</v>
+        <v>1128.32421875</v>
       </c>
       <c r="P41" t="n">
-        <v>25</v>
+        <v>11.4</v>
       </c>
       <c r="Q41" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R41" t="n">
         <v>0</v>
@@ -3129,7 +3209,7 @@
         <v>0</v>
       </c>
       <c r="T41" t="n">
-        <v>0.001933813095092773</v>
+        <v>22.51702928543091</v>
       </c>
       <c r="U41" t="n">
         <v>0</v>
@@ -3145,47 +3225,49 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>0.01273885288652687</v>
+        <v>0.2847457577165183</v>
       </c>
       <c r="D42" t="n">
-        <v>7.842246496009318e-255</v>
+        <v>8.80739104117219e-79</v>
       </c>
       <c r="E42" t="n">
-        <v>0.3200334906578064</v>
+        <v>0.5993292331695557</v>
       </c>
       <c r="F42" t="n">
-        <v>12.42500000000001</v>
+        <v>47.20628289473686</v>
       </c>
       <c r="G42" t="n">
-        <v>0.08114285714285714</v>
+        <v>0.8594285714285714</v>
       </c>
       <c r="H42" t="n">
-        <v>0</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="I42" t="n">
         <v>1</v>
       </c>
-      <c r="J42" t="inlineStr"/>
+      <c r="J42" t="n">
+        <v>1</v>
+      </c>
       <c r="K42" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L42" t="n">
         <v>0</v>
       </c>
       <c r="M42" t="n">
-        <v>0.1111111111111111</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="N42" t="n">
-        <v>0.002156734466552734</v>
+        <v>20.88469409942627</v>
       </c>
       <c r="O42" t="n">
-        <v>1122.859375</v>
+        <v>1128.32421875</v>
       </c>
       <c r="P42" t="n">
-        <v>0</v>
+        <v>11.6</v>
       </c>
       <c r="Q42" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R42" t="n">
         <v>0</v>
@@ -3194,7 +3276,7 @@
         <v>0</v>
       </c>
       <c r="T42" t="n">
-        <v>0.002155303955078125</v>
+        <v>20.88469219207764</v>
       </c>
       <c r="U42" t="n">
         <v>0</v>
@@ -3210,47 +3292,49 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>0</v>
+        <v>0.2078651635494257</v>
       </c>
       <c r="D43" t="n">
-        <v>0</v>
+        <v>7.851922773836407e-79</v>
       </c>
       <c r="E43" t="n">
-        <v>0.3462300896644592</v>
+        <v>0.6243407726287842</v>
       </c>
       <c r="F43" t="n">
-        <v>12.42500000000001</v>
+        <v>24.61820635136979</v>
       </c>
       <c r="G43" t="n">
-        <v>0.06580166821130677</v>
+        <v>1.034291010194625</v>
       </c>
       <c r="H43" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I43" t="n">
-        <v>0</v>
-      </c>
-      <c r="J43" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J43" t="n">
+        <v>0.6666666666666666</v>
+      </c>
       <c r="K43" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L43" t="n">
         <v>0</v>
       </c>
       <c r="M43" t="n">
-        <v>0.02439024390243903</v>
+        <v>0.1891891891891892</v>
       </c>
       <c r="N43" t="n">
-        <v>0.002086877822875977</v>
+        <v>22.19956421852112</v>
       </c>
       <c r="O43" t="n">
-        <v>1122.859375</v>
+        <v>1128.32421875</v>
       </c>
       <c r="P43" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="Q43" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R43" t="n">
         <v>0</v>
@@ -3259,7 +3343,7 @@
         <v>0</v>
       </c>
       <c r="T43" t="n">
-        <v>0.002085208892822266</v>
+        <v>22.19956254959106</v>
       </c>
       <c r="U43" t="n">
         <v>0</v>
@@ -3275,47 +3359,49 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>0</v>
+        <v>0.1831501783681521</v>
       </c>
       <c r="D44" t="n">
-        <v>0</v>
+        <v>5.32410154959273e-79</v>
       </c>
       <c r="E44" t="n">
-        <v>0.3189048171043396</v>
+        <v>0.6311661005020142</v>
       </c>
       <c r="F44" t="n">
-        <v>12.42500000000001</v>
+        <v>14.84206632653061</v>
       </c>
       <c r="G44" t="n">
-        <v>0.08151549942594719</v>
+        <v>0.7841561423650976</v>
       </c>
       <c r="H44" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="I44" t="n">
-        <v>0</v>
-      </c>
-      <c r="J44" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J44" t="n">
+        <v>1</v>
+      </c>
       <c r="K44" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L44" t="n">
         <v>0</v>
       </c>
       <c r="M44" t="n">
-        <v>0.06666666666666667</v>
+        <v>0.2105263157894737</v>
       </c>
       <c r="N44" t="n">
-        <v>0.002296924591064453</v>
+        <v>23.71668314933777</v>
       </c>
       <c r="O44" t="n">
-        <v>1122.859375</v>
+        <v>1128.32421875</v>
       </c>
       <c r="P44" t="n">
-        <v>0</v>
+        <v>11.3</v>
       </c>
       <c r="Q44" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R44" t="n">
         <v>0</v>
@@ -3324,7 +3410,7 @@
         <v>0</v>
       </c>
       <c r="T44" t="n">
-        <v>0.002295732498168945</v>
+        <v>23.7166805267334</v>
       </c>
       <c r="U44" t="n">
         <v>0</v>
@@ -3340,47 +3426,49 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>0</v>
+        <v>0.1313131289823034</v>
       </c>
       <c r="D45" t="n">
-        <v>0</v>
+        <v>2.328008250173485e-160</v>
       </c>
       <c r="E45" t="n">
-        <v>0.3425029814243317</v>
+        <v>0.5515757203102112</v>
       </c>
       <c r="F45" t="n">
-        <v>12.42500000000001</v>
+        <v>14.61376237623762</v>
       </c>
       <c r="G45" t="n">
-        <v>0.01946805593638607</v>
+        <v>0.1258568686591719</v>
       </c>
       <c r="H45" t="n">
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="I45" t="n">
         <v>0</v>
       </c>
-      <c r="J45" t="inlineStr"/>
+      <c r="J45" t="n">
+        <v>1</v>
+      </c>
       <c r="K45" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L45" t="n">
         <v>0</v>
       </c>
       <c r="M45" t="n">
-        <v>0.06666666666666667</v>
+        <v>0.1935483870967742</v>
       </c>
       <c r="N45" t="n">
-        <v>0.002425193786621094</v>
+        <v>30.68054127693176</v>
       </c>
       <c r="O45" t="n">
-        <v>1122.86328125</v>
+        <v>1128.32421875</v>
       </c>
       <c r="P45" t="n">
-        <v>0</v>
+        <v>11.4</v>
       </c>
       <c r="Q45" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R45" t="n">
         <v>0</v>
@@ -3389,7 +3477,7 @@
         <v>0</v>
       </c>
       <c r="T45" t="n">
-        <v>0.002423524856567383</v>
+        <v>30.68053936958313</v>
       </c>
       <c r="U45" t="n">
         <v>0</v>
@@ -3405,47 +3493,49 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>0</v>
+        <v>0.3433813851825844</v>
       </c>
       <c r="D46" t="n">
-        <v>0</v>
+        <v>0.04451783982059418</v>
       </c>
       <c r="E46" t="n">
-        <v>0.3373959362506866</v>
+        <v>0.6453493237495422</v>
       </c>
       <c r="F46" t="n">
-        <v>12.42500000000001</v>
+        <v>56.65225684931511</v>
       </c>
       <c r="G46" t="n">
-        <v>0.01966214345056771</v>
+        <v>0.3793962891165882</v>
       </c>
       <c r="H46" t="n">
-        <v>0</v>
+        <v>0.7142857142857143</v>
       </c>
       <c r="I46" t="n">
-        <v>0</v>
-      </c>
-      <c r="J46" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J46" t="n">
+        <v>1</v>
+      </c>
       <c r="K46" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L46" t="n">
         <v>0</v>
       </c>
       <c r="M46" t="n">
-        <v>0.1111111111111111</v>
+        <v>0.5714285714285714</v>
       </c>
       <c r="N46" t="n">
-        <v>0.002283334732055664</v>
+        <v>28.15051794052124</v>
       </c>
       <c r="O46" t="n">
-        <v>1122.86328125</v>
+        <v>1128.32421875</v>
       </c>
       <c r="P46" t="n">
-        <v>25</v>
+        <v>11.8</v>
       </c>
       <c r="Q46" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R46" t="n">
         <v>0</v>
@@ -3454,7 +3544,7 @@
         <v>0</v>
       </c>
       <c r="T46" t="n">
-        <v>0.002282142639160156</v>
+        <v>28.15051627159119</v>
       </c>
       <c r="U46" t="n">
         <v>0</v>
@@ -3470,27 +3560,29 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>0</v>
+        <v>0.2185566976151345</v>
       </c>
       <c r="D47" t="n">
-        <v>0</v>
+        <v>0.0001941507012433737</v>
       </c>
       <c r="E47" t="n">
-        <v>0.358601450920105</v>
+        <v>0.610046923160553</v>
       </c>
       <c r="F47" t="n">
-        <v>12.42500000000001</v>
+        <v>22.5976737967915</v>
       </c>
       <c r="G47" t="n">
-        <v>0.0282981267437226</v>
+        <v>0.2287764049422081</v>
       </c>
       <c r="H47" t="n">
-        <v>0</v>
+        <v>0.4285714285714285</v>
       </c>
       <c r="I47" t="n">
-        <v>0</v>
-      </c>
-      <c r="J47" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J47" t="n">
+        <v>1</v>
+      </c>
       <c r="K47" t="n">
         <v>0</v>
       </c>
@@ -3498,19 +3590,19 @@
         <v>0</v>
       </c>
       <c r="M47" t="n">
-        <v>0.07692307692307693</v>
+        <v>0.2156862745098039</v>
       </c>
       <c r="N47" t="n">
-        <v>0.002351284027099609</v>
+        <v>27.06231689453125</v>
       </c>
       <c r="O47" t="n">
-        <v>1122.86328125</v>
+        <v>1128.32421875</v>
       </c>
       <c r="P47" t="n">
-        <v>0</v>
+        <v>10.9</v>
       </c>
       <c r="Q47" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R47" t="n">
         <v>0</v>
@@ -3519,7 +3611,7 @@
         <v>0</v>
       </c>
       <c r="T47" t="n">
-        <v>0.002350330352783203</v>
+        <v>27.0623152256012</v>
       </c>
       <c r="U47" t="n">
         <v>0</v>
@@ -3535,47 +3627,49 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>0</v>
+        <v>0.2307692261316569</v>
       </c>
       <c r="D48" t="n">
-        <v>0</v>
+        <v>4.204956870067577e-155</v>
       </c>
       <c r="E48" t="n">
-        <v>0.3561545312404633</v>
+        <v>0.624326765537262</v>
       </c>
       <c r="F48" t="n">
-        <v>12.42500000000001</v>
+        <v>34.48713815789478</v>
       </c>
       <c r="G48" t="n">
-        <v>0.15203426124197</v>
+        <v>1.644539614561028</v>
       </c>
       <c r="H48" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="I48" t="n">
-        <v>0</v>
-      </c>
-      <c r="J48" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J48" t="n">
+        <v>1</v>
+      </c>
       <c r="K48" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L48" t="n">
         <v>0</v>
       </c>
       <c r="M48" t="n">
-        <v>0.06666666666666667</v>
+        <v>0.2660550458715596</v>
       </c>
       <c r="N48" t="n">
-        <v>0.001970052719116211</v>
+        <v>20.33850884437561</v>
       </c>
       <c r="O48" t="n">
-        <v>1122.86328125</v>
+        <v>1128.32421875</v>
       </c>
       <c r="P48" t="n">
-        <v>0</v>
+        <v>10.7</v>
       </c>
       <c r="Q48" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R48" t="n">
         <v>0</v>
@@ -3584,7 +3678,7 @@
         <v>0</v>
       </c>
       <c r="T48" t="n">
-        <v>0.001969099044799805</v>
+        <v>20.33850693702698</v>
       </c>
       <c r="U48" t="n">
         <v>0</v>
@@ -3600,47 +3694,49 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>0</v>
+        <v>0.2713567789863893</v>
       </c>
       <c r="D49" t="n">
-        <v>0</v>
+        <v>1.035880491824639e-78</v>
       </c>
       <c r="E49" t="n">
-        <v>0.3449079990386963</v>
+        <v>0.6271861791610718</v>
       </c>
       <c r="F49" t="n">
-        <v>12.42500000000001</v>
+        <v>44.44180555555556</v>
       </c>
       <c r="G49" t="n">
-        <v>0.1368015414258189</v>
+        <v>1.18111753371869</v>
       </c>
       <c r="H49" t="n">
-        <v>0</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="I49" t="n">
-        <v>0</v>
-      </c>
-      <c r="J49" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J49" t="n">
+        <v>1</v>
+      </c>
       <c r="K49" t="n">
-        <v>0</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="L49" t="n">
         <v>0</v>
       </c>
       <c r="M49" t="n">
-        <v>0.06666666666666667</v>
+        <v>0.2241379310344828</v>
       </c>
       <c r="N49" t="n">
-        <v>0.002166032791137695</v>
+        <v>22.48460125923157</v>
       </c>
       <c r="O49" t="n">
-        <v>1122.86328125</v>
+        <v>1128.32421875</v>
       </c>
       <c r="P49" t="n">
-        <v>25</v>
+        <v>11.8</v>
       </c>
       <c r="Q49" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R49" t="n">
         <v>0</v>
@@ -3649,7 +3745,7 @@
         <v>0</v>
       </c>
       <c r="T49" t="n">
-        <v>0.002164602279663086</v>
+        <v>22.48459911346436</v>
       </c>
       <c r="U49" t="n">
         <v>0</v>
@@ -3665,47 +3761,49 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>0</v>
+        <v>0.1991701198450441</v>
       </c>
       <c r="D50" t="n">
-        <v>0</v>
+        <v>7.642947701111475e-79</v>
       </c>
       <c r="E50" t="n">
-        <v>0.3456511199474335</v>
+        <v>0.5884968638420105</v>
       </c>
       <c r="F50" t="n">
-        <v>12.42500000000001</v>
+        <v>34.50517605633806</v>
       </c>
       <c r="G50" t="n">
-        <v>0.1360153256704981</v>
+        <v>1.580459770114943</v>
       </c>
       <c r="H50" t="n">
-        <v>0</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="I50" t="n">
-        <v>0</v>
-      </c>
-      <c r="J50" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J50" t="n">
+        <v>1</v>
+      </c>
       <c r="K50" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L50" t="n">
         <v>0</v>
       </c>
       <c r="M50" t="n">
-        <v>0.06666666666666667</v>
+        <v>0.2105263157894737</v>
       </c>
       <c r="N50" t="n">
-        <v>0.001978635787963867</v>
+        <v>22.73816633224487</v>
       </c>
       <c r="O50" t="n">
-        <v>1122.86328125</v>
+        <v>1128.32421875</v>
       </c>
       <c r="P50" t="n">
-        <v>25</v>
+        <v>11.3</v>
       </c>
       <c r="Q50" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R50" t="n">
         <v>0</v>
@@ -3714,7 +3812,7 @@
         <v>0</v>
       </c>
       <c r="T50" t="n">
-        <v>0.001977205276489258</v>
+        <v>22.73816418647766</v>
       </c>
       <c r="U50" t="n">
         <v>0</v>
@@ -3730,47 +3828,49 @@
         </is>
       </c>
       <c r="C51" t="n">
-        <v>0</v>
+        <v>0.2687746985611399</v>
       </c>
       <c r="D51" t="n">
-        <v>0</v>
+        <v>0.02181214498771713</v>
       </c>
       <c r="E51" t="n">
-        <v>0.3437384366989136</v>
+        <v>0.6134772896766663</v>
       </c>
       <c r="F51" t="n">
-        <v>12.42500000000001</v>
+        <v>22.84828627572657</v>
       </c>
       <c r="G51" t="n">
-        <v>0.09454061251664447</v>
+        <v>1.22237017310253</v>
       </c>
       <c r="H51" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I51" t="n">
-        <v>0</v>
-      </c>
-      <c r="J51" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J51" t="n">
+        <v>0</v>
+      </c>
       <c r="K51" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L51" t="n">
         <v>0</v>
       </c>
       <c r="M51" t="n">
-        <v>0.07692307692307693</v>
+        <v>0.5</v>
       </c>
       <c r="N51" t="n">
-        <v>0.002255439758300781</v>
+        <v>26.77148342132568</v>
       </c>
       <c r="O51" t="n">
-        <v>1122.86328125</v>
+        <v>1128.32421875</v>
       </c>
       <c r="P51" t="n">
-        <v>0</v>
+        <v>11.3</v>
       </c>
       <c r="Q51" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R51" t="n">
         <v>0</v>
@@ -3779,7 +3879,7 @@
         <v>0</v>
       </c>
       <c r="T51" t="n">
-        <v>0.002254486083984375</v>
+        <v>26.77148079872131</v>
       </c>
       <c r="U51" t="n">
         <v>0</v>
@@ -3795,47 +3895,49 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>0.008403360933196829</v>
+        <v>0.1941176427455018</v>
       </c>
       <c r="D52" t="n">
-        <v>2.960553565183628e-265</v>
+        <v>0.009029607958494362</v>
       </c>
       <c r="E52" t="n">
-        <v>0.3465096652507782</v>
+        <v>0.5965020060539246</v>
       </c>
       <c r="F52" t="n">
-        <v>12.42500000000001</v>
+        <v>31.85625000000002</v>
       </c>
       <c r="G52" t="n">
-        <v>0.05148658448150834</v>
+        <v>0.4263959390862944</v>
       </c>
       <c r="H52" t="n">
-        <v>0</v>
+        <v>0.1666666666666667</v>
       </c>
       <c r="I52" t="n">
-        <v>0</v>
-      </c>
-      <c r="J52" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J52" t="n">
+        <v>1</v>
+      </c>
       <c r="K52" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="L52" t="n">
         <v>0</v>
       </c>
       <c r="M52" t="n">
-        <v>0.09090909090909091</v>
+        <v>0.2134831460674157</v>
       </c>
       <c r="N52" t="n">
-        <v>0.002103090286254883</v>
+        <v>23.46485590934753</v>
       </c>
       <c r="O52" t="n">
-        <v>1122.87109375</v>
+        <v>1128.32421875</v>
       </c>
       <c r="P52" t="n">
-        <v>0</v>
+        <v>11.6</v>
       </c>
       <c r="Q52" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R52" t="n">
         <v>0</v>
@@ -3844,7 +3946,7 @@
         <v>0</v>
       </c>
       <c r="T52" t="n">
-        <v>0.002101421356201172</v>
+        <v>23.46485304832458</v>
       </c>
       <c r="U52" t="n">
         <v>0</v>
@@ -3860,27 +3962,29 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>0</v>
+        <v>0.1588235269448097</v>
       </c>
       <c r="D53" t="n">
-        <v>0</v>
+        <v>2.876839432916431e-05</v>
       </c>
       <c r="E53" t="n">
-        <v>0.3215235471725464</v>
+        <v>0.5168488025665283</v>
       </c>
       <c r="F53" t="n">
-        <v>12.42500000000001</v>
+        <v>25.57649647887325</v>
       </c>
       <c r="G53" t="n">
-        <v>0.03788687299893276</v>
+        <v>0.1616862326574173</v>
       </c>
       <c r="H53" t="n">
         <v>0</v>
       </c>
       <c r="I53" t="n">
-        <v>0</v>
-      </c>
-      <c r="J53" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J53" t="n">
+        <v>1</v>
+      </c>
       <c r="K53" t="n">
         <v>0</v>
       </c>
@@ -3888,19 +3992,19 @@
         <v>0</v>
       </c>
       <c r="M53" t="n">
-        <v>0.04761904761904762</v>
+        <v>0.0728476821192053</v>
       </c>
       <c r="N53" t="n">
-        <v>0.002568721771240234</v>
+        <v>27.59025812149048</v>
       </c>
       <c r="O53" t="n">
-        <v>1122.90625</v>
+        <v>1128.32421875</v>
       </c>
       <c r="P53" t="n">
-        <v>0</v>
+        <v>10.9</v>
       </c>
       <c r="Q53" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R53" t="n">
         <v>0</v>
@@ -3909,7 +4013,7 @@
         <v>0</v>
       </c>
       <c r="T53" t="n">
-        <v>0.002567291259765625</v>
+        <v>27.59025597572327</v>
       </c>
       <c r="U53" t="n">
         <v>0</v>
@@ -3925,47 +4029,49 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>0</v>
+        <v>0.2090395431759713</v>
       </c>
       <c r="D54" t="n">
-        <v>0</v>
+        <v>2.084042041730364e-79</v>
       </c>
       <c r="E54" t="n">
-        <v>0.3136659562587738</v>
+        <v>0.6238571405410767</v>
       </c>
       <c r="F54" t="n">
-        <v>12.42500000000001</v>
+        <v>0.5445535714285938</v>
       </c>
       <c r="G54" t="n">
-        <v>0.05224429727740986</v>
+        <v>0.6600441501103753</v>
       </c>
       <c r="H54" t="n">
-        <v>0</v>
+        <v>0.4545454545454545</v>
       </c>
       <c r="I54" t="n">
-        <v>0</v>
-      </c>
-      <c r="J54" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J54" t="n">
+        <v>1</v>
+      </c>
       <c r="K54" t="n">
-        <v>0</v>
+        <v>0.75</v>
       </c>
       <c r="L54" t="n">
         <v>0</v>
       </c>
       <c r="M54" t="n">
-        <v>0.06666666666666667</v>
+        <v>0.2622950819672131</v>
       </c>
       <c r="N54" t="n">
-        <v>0.002014398574829102</v>
+        <v>26.47705173492432</v>
       </c>
       <c r="O54" t="n">
-        <v>1122.90625</v>
+        <v>1128.32421875</v>
       </c>
       <c r="P54" t="n">
-        <v>33.3</v>
+        <v>11.3</v>
       </c>
       <c r="Q54" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R54" t="n">
         <v>0</v>
@@ -3974,7 +4080,7 @@
         <v>0</v>
       </c>
       <c r="T54" t="n">
-        <v>0.002013683319091797</v>
+        <v>26.47704982757568</v>
       </c>
       <c r="U54" t="n">
         <v>0</v>
@@ -3990,47 +4096,49 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>0</v>
+        <v>0.2412868586089169</v>
       </c>
       <c r="D55" t="n">
-        <v>0</v>
+        <v>6.245369322936759e-156</v>
       </c>
       <c r="E55" t="n">
-        <v>0.3323594033718109</v>
+        <v>0.6119844317436218</v>
       </c>
       <c r="F55" t="n">
-        <v>12.42500000000001</v>
+        <v>33.69093548387099</v>
       </c>
       <c r="G55" t="n">
-        <v>0.04592496765847348</v>
+        <v>0.4695989650711513</v>
       </c>
       <c r="H55" t="n">
-        <v>0</v>
+        <v>0.2105263157894737</v>
       </c>
       <c r="I55" t="n">
-        <v>0</v>
-      </c>
-      <c r="J55" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J55" t="n">
+        <v>1</v>
+      </c>
       <c r="K55" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L55" t="n">
         <v>0</v>
       </c>
       <c r="M55" t="n">
-        <v>0.09090909090909091</v>
+        <v>0.2156862745098039</v>
       </c>
       <c r="N55" t="n">
-        <v>0.0021820068359375</v>
+        <v>23.25298380851746</v>
       </c>
       <c r="O55" t="n">
-        <v>1122.91015625</v>
+        <v>1128.32421875</v>
       </c>
       <c r="P55" t="n">
-        <v>0</v>
+        <v>11.6</v>
       </c>
       <c r="Q55" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R55" t="n">
         <v>0</v>
@@ -4039,7 +4147,7 @@
         <v>0</v>
       </c>
       <c r="T55" t="n">
-        <v>0.002180814743041992</v>
+        <v>23.25298190116882</v>
       </c>
       <c r="U55" t="n">
         <v>0</v>
@@ -4055,47 +4163,49 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>0</v>
+        <v>0.1971014452331864</v>
       </c>
       <c r="D56" t="n">
-        <v>0</v>
+        <v>2.626892551353189e-80</v>
       </c>
       <c r="E56" t="n">
-        <v>0.315963089466095</v>
+        <v>0.5822121500968933</v>
       </c>
       <c r="F56" t="n">
-        <v>12.42500000000001</v>
+        <v>17.59505376344089</v>
       </c>
       <c r="G56" t="n">
-        <v>0.04530950861518826</v>
+        <v>0.364390555201021</v>
       </c>
       <c r="H56" t="n">
-        <v>0</v>
+        <v>0.04761904761904762</v>
       </c>
       <c r="I56" t="n">
         <v>0</v>
       </c>
-      <c r="J56" t="inlineStr"/>
+      <c r="J56" t="n">
+        <v>1</v>
+      </c>
       <c r="K56" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="L56" t="n">
         <v>0</v>
       </c>
       <c r="M56" t="n">
-        <v>0.09090909090909091</v>
+        <v>0.2941176470588235</v>
       </c>
       <c r="N56" t="n">
-        <v>0.001950263977050781</v>
+        <v>21.16882419586182</v>
       </c>
       <c r="O56" t="n">
-        <v>1122.91015625</v>
+        <v>1128.32421875</v>
       </c>
       <c r="P56" t="n">
-        <v>0</v>
+        <v>10.9</v>
       </c>
       <c r="Q56" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R56" t="n">
         <v>0</v>
@@ -4104,7 +4214,7 @@
         <v>0</v>
       </c>
       <c r="T56" t="n">
-        <v>0.001949548721313477</v>
+        <v>21.16882228851318</v>
       </c>
       <c r="U56" t="n">
         <v>0</v>
@@ -4120,47 +4230,49 @@
         </is>
       </c>
       <c r="C57" t="n">
-        <v>0</v>
+        <v>0.181818178462272</v>
       </c>
       <c r="D57" t="n">
-        <v>0</v>
+        <v>1.153567111099626e-80</v>
       </c>
       <c r="E57" t="n">
-        <v>0.3651198446750641</v>
+        <v>0.5616248250007629</v>
       </c>
       <c r="F57" t="n">
-        <v>12.42500000000001</v>
+        <v>23.91363636363641</v>
       </c>
       <c r="G57" t="n">
-        <v>0.02446588559614059</v>
+        <v>0.2467263955892488</v>
       </c>
       <c r="H57" t="n">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="I57" t="n">
-        <v>0</v>
-      </c>
-      <c r="J57" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J57" t="n">
+        <v>0</v>
+      </c>
       <c r="K57" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L57" t="n">
         <v>0</v>
       </c>
       <c r="M57" t="n">
-        <v>0.03703703703703703</v>
+        <v>0.2432432432432433</v>
       </c>
       <c r="N57" t="n">
-        <v>0.002827644348144531</v>
+        <v>32.27656555175781</v>
       </c>
       <c r="O57" t="n">
-        <v>1122.9296875</v>
+        <v>1128.37109375</v>
       </c>
       <c r="P57" t="n">
-        <v>20</v>
+        <v>11.2</v>
       </c>
       <c r="Q57" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R57" t="n">
         <v>0</v>
@@ -4169,7 +4281,7 @@
         <v>0</v>
       </c>
       <c r="T57" t="n">
-        <v>0.002826213836669922</v>
+        <v>32.2765634059906</v>
       </c>
       <c r="U57" t="n">
         <v>0</v>
@@ -4185,47 +4297,49 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>0.0120481921868196</v>
+        <v>0.1634241198334571</v>
       </c>
       <c r="D58" t="n">
-        <v>3.542014107114671e-257</v>
+        <v>9.10883278677377e-156</v>
       </c>
       <c r="E58" t="n">
-        <v>0.3421286642551422</v>
+        <v>0.5662688612937927</v>
       </c>
       <c r="F58" t="n">
-        <v>12.42500000000001</v>
+        <v>15.26577922077925</v>
       </c>
       <c r="G58" t="n">
-        <v>0.07667386609071274</v>
+        <v>0.6015118790496761</v>
       </c>
       <c r="H58" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="I58" t="n">
-        <v>0</v>
-      </c>
-      <c r="J58" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J58" t="n">
+        <v>1</v>
+      </c>
       <c r="K58" t="n">
-        <v>0</v>
+        <v>0.875</v>
       </c>
       <c r="L58" t="n">
         <v>0</v>
       </c>
       <c r="M58" t="n">
-        <v>0.1111111111111111</v>
+        <v>0.1666666666666667</v>
       </c>
       <c r="N58" t="n">
-        <v>0.002401113510131836</v>
+        <v>19.19828152656555</v>
       </c>
       <c r="O58" t="n">
-        <v>1122.9375</v>
+        <v>1128.37109375</v>
       </c>
       <c r="P58" t="n">
-        <v>0</v>
+        <v>11.3</v>
       </c>
       <c r="Q58" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R58" t="n">
         <v>0</v>
@@ -4234,7 +4348,7 @@
         <v>0</v>
       </c>
       <c r="T58" t="n">
-        <v>0.002399444580078125</v>
+        <v>19.19827938079834</v>
       </c>
       <c r="U58" t="n">
         <v>0</v>
@@ -4250,47 +4364,49 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>0</v>
+        <v>0.0978260827221174</v>
       </c>
       <c r="D59" t="n">
-        <v>0</v>
+        <v>1.502178278808791e-232</v>
       </c>
       <c r="E59" t="n">
-        <v>0.365123987197876</v>
+        <v>0.5114860534667969</v>
       </c>
       <c r="F59" t="n">
-        <v>12.42500000000001</v>
+        <v>23.51032608695655</v>
       </c>
       <c r="G59" t="n">
-        <v>0.08964646464646464</v>
+        <v>0.4419191919191919</v>
       </c>
       <c r="H59" t="n">
         <v>0</v>
       </c>
       <c r="I59" t="n">
-        <v>0</v>
-      </c>
-      <c r="J59" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J59" t="n">
+        <v>1</v>
+      </c>
       <c r="K59" t="n">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="L59" t="n">
         <v>0</v>
       </c>
       <c r="M59" t="n">
-        <v>0.09090909090909091</v>
+        <v>0.1428571428571428</v>
       </c>
       <c r="N59" t="n">
-        <v>0.002303361892700195</v>
+        <v>25.09474587440491</v>
       </c>
       <c r="O59" t="n">
-        <v>1122.9375</v>
+        <v>1128.37109375</v>
       </c>
       <c r="P59" t="n">
-        <v>0</v>
+        <v>11.1</v>
       </c>
       <c r="Q59" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R59" t="n">
         <v>0</v>
@@ -4299,7 +4415,7 @@
         <v>0</v>
       </c>
       <c r="T59" t="n">
-        <v>0.002301692962646484</v>
+        <v>25.09474396705627</v>
       </c>
       <c r="U59" t="n">
         <v>0</v>
@@ -4315,27 +4431,29 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>0.00446428549356267</v>
+        <v>0.1699819136304034</v>
       </c>
       <c r="D60" t="n">
-        <v>8.265132997605698e-314</v>
+        <v>1.059108558790827e-80</v>
       </c>
       <c r="E60" t="n">
-        <v>0.3449465930461884</v>
+        <v>0.5727046132087708</v>
       </c>
       <c r="F60" t="n">
-        <v>12.42500000000001</v>
+        <v>31.1515</v>
       </c>
       <c r="G60" t="n">
-        <v>0.02480782669461915</v>
+        <v>0.2124388539482879</v>
       </c>
       <c r="H60" t="n">
-        <v>0</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="I60" t="n">
-        <v>0</v>
-      </c>
-      <c r="J60" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J60" t="n">
+        <v>1</v>
+      </c>
       <c r="K60" t="n">
         <v>0</v>
       </c>
@@ -4343,19 +4461,19 @@
         <v>0</v>
       </c>
       <c r="M60" t="n">
-        <v>0.06666666666666667</v>
+        <v>0.2</v>
       </c>
       <c r="N60" t="n">
-        <v>0.002183198928833008</v>
+        <v>27.59090447425842</v>
       </c>
       <c r="O60" t="n">
-        <v>1122.95703125</v>
+        <v>1128.37109375</v>
       </c>
       <c r="P60" t="n">
-        <v>0</v>
+        <v>11.6</v>
       </c>
       <c r="Q60" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R60" t="n">
         <v>0</v>
@@ -4364,7 +4482,7 @@
         <v>0</v>
       </c>
       <c r="T60" t="n">
-        <v>0.002181768417358398</v>
+        <v>27.59090232849121</v>
       </c>
       <c r="U60" t="n">
         <v>0</v>
@@ -4380,47 +4498,49 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>0</v>
+        <v>0.1694915217164609</v>
       </c>
       <c r="D61" t="n">
-        <v>0</v>
+        <v>2.641122902589137e-155</v>
       </c>
       <c r="E61" t="n">
-        <v>0.3740620315074921</v>
+        <v>0.4670159816741943</v>
       </c>
       <c r="F61" t="n">
-        <v>12.42500000000001</v>
+        <v>42.60887931034486</v>
       </c>
       <c r="G61" t="n">
-        <v>0.2874493927125506</v>
+        <v>1.983805668016194</v>
       </c>
       <c r="H61" t="n">
         <v>1</v>
       </c>
       <c r="I61" t="n">
-        <v>0</v>
-      </c>
-      <c r="J61" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J61" t="n">
+        <v>1</v>
+      </c>
       <c r="K61" t="n">
-        <v>0</v>
+        <v>0.975</v>
       </c>
       <c r="L61" t="n">
         <v>0</v>
       </c>
       <c r="M61" t="n">
-        <v>0.05263157894736842</v>
+        <v>0.1240875912408759</v>
       </c>
       <c r="N61" t="n">
-        <v>0.002161502838134766</v>
+        <v>24.68773412704468</v>
       </c>
       <c r="O61" t="n">
-        <v>1122.95703125</v>
+        <v>1128.37109375</v>
       </c>
       <c r="P61" t="n">
-        <v>25</v>
+        <v>11.2</v>
       </c>
       <c r="Q61" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R61" t="n">
         <v>0</v>
@@ -4429,7 +4549,7 @@
         <v>0</v>
       </c>
       <c r="T61" t="n">
-        <v>0.002160310745239258</v>
+        <v>24.68773198127747</v>
       </c>
       <c r="U61" t="n">
         <v>0</v>
@@ -4445,47 +4565,49 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>0</v>
+        <v>0.159663861293341</v>
       </c>
       <c r="D62" t="n">
-        <v>0</v>
+        <v>2.360787777620462e-155</v>
       </c>
       <c r="E62" t="n">
-        <v>0.3254433572292328</v>
+        <v>0.5814318060874939</v>
       </c>
       <c r="F62" t="n">
-        <v>12.42500000000001</v>
+        <v>34.4511641791045</v>
       </c>
       <c r="G62" t="n">
-        <v>0.1775</v>
+        <v>2.44</v>
       </c>
       <c r="H62" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I62" t="n">
-        <v>0</v>
-      </c>
-      <c r="J62" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J62" t="n">
+        <v>1</v>
+      </c>
       <c r="K62" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L62" t="n">
         <v>0</v>
       </c>
       <c r="M62" t="n">
-        <v>0.06666666666666667</v>
+        <v>0.2307692307692308</v>
       </c>
       <c r="N62" t="n">
-        <v>0.001862525939941406</v>
+        <v>18.8063759803772</v>
       </c>
       <c r="O62" t="n">
-        <v>1122.95703125</v>
+        <v>1128.37109375</v>
       </c>
       <c r="P62" t="n">
-        <v>0</v>
+        <v>10.6</v>
       </c>
       <c r="Q62" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R62" t="n">
         <v>0</v>
@@ -4494,7 +4616,7 @@
         <v>0</v>
       </c>
       <c r="T62" t="n">
-        <v>0.001861572265625</v>
+        <v>18.80637407302856</v>
       </c>
       <c r="U62" t="n">
         <v>0</v>
@@ -4510,27 +4632,29 @@
         </is>
       </c>
       <c r="C63" t="n">
-        <v>0</v>
+        <v>0.2472727222780827</v>
       </c>
       <c r="D63" t="n">
-        <v>0</v>
+        <v>4.252812121486095e-155</v>
       </c>
       <c r="E63" t="n">
-        <v>0.3147302865982056</v>
+        <v>0.5911986231803894</v>
       </c>
       <c r="F63" t="n">
-        <v>12.42500000000001</v>
+        <v>42.45704736547088</v>
       </c>
       <c r="G63" t="n">
-        <v>0.09902370990237098</v>
+        <v>1.118549511854951</v>
       </c>
       <c r="H63" t="n">
-        <v>0</v>
+        <v>0.75</v>
       </c>
       <c r="I63" t="n">
-        <v>0</v>
-      </c>
-      <c r="J63" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J63" t="n">
+        <v>1</v>
+      </c>
       <c r="K63" t="n">
         <v>0</v>
       </c>
@@ -4538,19 +4662,19 @@
         <v>0</v>
       </c>
       <c r="M63" t="n">
-        <v>0.06666666666666667</v>
+        <v>0.2380952380952381</v>
       </c>
       <c r="N63" t="n">
-        <v>0.002123355865478516</v>
+        <v>20.03243947029114</v>
       </c>
       <c r="O63" t="n">
-        <v>1122.95703125</v>
+        <v>1128.37109375</v>
       </c>
       <c r="P63" t="n">
-        <v>0</v>
+        <v>11.9</v>
       </c>
       <c r="Q63" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R63" t="n">
         <v>0</v>
@@ -4559,7 +4683,7 @@
         <v>0</v>
       </c>
       <c r="T63" t="n">
-        <v>0.002121925354003906</v>
+        <v>20.03243780136108</v>
       </c>
       <c r="U63" t="n">
         <v>0</v>
@@ -4575,47 +4699,49 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>0</v>
+        <v>0.2327586157030322</v>
       </c>
       <c r="D64" t="n">
-        <v>0</v>
+        <v>0.02405625328689112</v>
       </c>
       <c r="E64" t="n">
-        <v>0.310442179441452</v>
+        <v>0.5778536796569824</v>
       </c>
       <c r="F64" t="n">
-        <v>12.42500000000001</v>
+        <v>21.71871273712742</v>
       </c>
       <c r="G64" t="n">
-        <v>0.1163934426229508</v>
+        <v>1.132786885245902</v>
       </c>
       <c r="H64" t="n">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="I64" t="n">
-        <v>0</v>
-      </c>
-      <c r="J64" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J64" t="n">
+        <v>1</v>
+      </c>
       <c r="K64" t="n">
-        <v>0</v>
+        <v>0.9166666666666666</v>
       </c>
       <c r="L64" t="n">
         <v>0</v>
       </c>
       <c r="M64" t="n">
-        <v>0.06666666666666667</v>
+        <v>0.186046511627907</v>
       </c>
       <c r="N64" t="n">
-        <v>0.002099990844726562</v>
+        <v>19.39385914802551</v>
       </c>
       <c r="O64" t="n">
-        <v>1122.95703125</v>
+        <v>1128.37109375</v>
       </c>
       <c r="P64" t="n">
-        <v>0</v>
+        <v>10.7</v>
       </c>
       <c r="Q64" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R64" t="n">
         <v>0</v>
@@ -4624,7 +4750,7 @@
         <v>0</v>
       </c>
       <c r="T64" t="n">
-        <v>0.002098560333251953</v>
+        <v>19.39385771751404</v>
       </c>
       <c r="U64" t="n">
         <v>0</v>
@@ -4640,47 +4766,49 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>0</v>
+        <v>0.1810344779384662</v>
       </c>
       <c r="D65" t="n">
-        <v>0</v>
+        <v>8.109369275808355e-79</v>
       </c>
       <c r="E65" t="n">
-        <v>0.3207126259803772</v>
+        <v>0.567719042301178</v>
       </c>
       <c r="F65" t="n">
-        <v>12.42500000000001</v>
+        <v>28.33250000000004</v>
       </c>
       <c r="G65" t="n">
-        <v>0.1422845691382766</v>
+        <v>1.543086172344689</v>
       </c>
       <c r="H65" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I65" t="n">
-        <v>0</v>
-      </c>
-      <c r="J65" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J65" t="n">
+        <v>1</v>
+      </c>
       <c r="K65" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L65" t="n">
         <v>0</v>
       </c>
       <c r="M65" t="n">
-        <v>0.06666666666666667</v>
+        <v>0.1509433962264151</v>
       </c>
       <c r="N65" t="n">
-        <v>0.001873016357421875</v>
+        <v>19.84823608398438</v>
       </c>
       <c r="O65" t="n">
-        <v>1122.95703125</v>
+        <v>1128.37109375</v>
       </c>
       <c r="P65" t="n">
-        <v>0</v>
+        <v>11.5</v>
       </c>
       <c r="Q65" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R65" t="n">
         <v>0</v>
@@ -4689,7 +4817,7 @@
         <v>0</v>
       </c>
       <c r="T65" t="n">
-        <v>0.001872062683105469</v>
+        <v>19.84823441505432</v>
       </c>
       <c r="U65" t="n">
         <v>0</v>
@@ -4705,47 +4833,49 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>0</v>
+        <v>0.2509803872861208</v>
       </c>
       <c r="D66" t="n">
-        <v>0</v>
+        <v>6.261661583609849e-79</v>
       </c>
       <c r="E66" t="n">
-        <v>0.3186623752117157</v>
+        <v>0.5955936908721924</v>
       </c>
       <c r="F66" t="n">
-        <v>12.42500000000001</v>
+        <v>33.91318987341774</v>
       </c>
       <c r="G66" t="n">
-        <v>0.0890840652446675</v>
+        <v>0.7540777917189461</v>
       </c>
       <c r="H66" t="n">
-        <v>0</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="I66" t="n">
-        <v>0</v>
-      </c>
-      <c r="J66" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J66" t="n">
+        <v>1</v>
+      </c>
       <c r="K66" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L66" t="n">
         <v>0</v>
       </c>
       <c r="M66" t="n">
-        <v>0.06666666666666667</v>
+        <v>0.148936170212766</v>
       </c>
       <c r="N66" t="n">
-        <v>0.002179861068725586</v>
+        <v>19.46893239021301</v>
       </c>
       <c r="O66" t="n">
-        <v>1122.95703125</v>
+        <v>1128.37109375</v>
       </c>
       <c r="P66" t="n">
-        <v>25</v>
+        <v>10.7</v>
       </c>
       <c r="Q66" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R66" t="n">
         <v>0</v>
@@ -4754,7 +4884,7 @@
         <v>0</v>
       </c>
       <c r="T66" t="n">
-        <v>0.00217890739440918</v>
+        <v>19.46893072128296</v>
       </c>
       <c r="U66" t="n">
         <v>0</v>
@@ -4770,47 +4900,49 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>0</v>
+        <v>0.2328767074047665</v>
       </c>
       <c r="D67" t="n">
-        <v>0</v>
+        <v>4.015646547179402e-155</v>
       </c>
       <c r="E67" t="n">
-        <v>0.3204876482486725</v>
+        <v>0.6221136450767517</v>
       </c>
       <c r="F67" t="n">
-        <v>12.42500000000001</v>
+        <v>43.80500000000004</v>
       </c>
       <c r="G67" t="n">
-        <v>0.09726027397260274</v>
+        <v>1.306849315068493</v>
       </c>
       <c r="H67" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="I67" t="n">
-        <v>0</v>
-      </c>
-      <c r="J67" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J67" t="n">
+        <v>1</v>
+      </c>
       <c r="K67" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L67" t="n">
         <v>0</v>
       </c>
       <c r="M67" t="n">
-        <v>0.06666666666666667</v>
+        <v>0.3396226415094339</v>
       </c>
       <c r="N67" t="n">
-        <v>0.001979827880859375</v>
+        <v>23.98936676979065</v>
       </c>
       <c r="O67" t="n">
-        <v>1122.95703125</v>
+        <v>1128.37109375</v>
       </c>
       <c r="P67" t="n">
-        <v>0</v>
+        <v>11.5</v>
       </c>
       <c r="Q67" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R67" t="n">
         <v>0</v>
@@ -4819,7 +4951,7 @@
         <v>0</v>
       </c>
       <c r="T67" t="n">
-        <v>0.001978874206542969</v>
+        <v>23.98936486244202</v>
       </c>
       <c r="U67" t="n">
         <v>0</v>
@@ -4835,47 +4967,49 @@
         </is>
       </c>
       <c r="C68" t="n">
-        <v>0</v>
+        <v>0.09259259020061734</v>
       </c>
       <c r="D68" t="n">
-        <v>0</v>
+        <v>8.06798322521923e-232</v>
       </c>
       <c r="E68" t="n">
-        <v>0.3620995283126831</v>
+        <v>0.4935102164745331</v>
       </c>
       <c r="F68" t="n">
-        <v>12.42500000000001</v>
+        <v>9.262820329277048</v>
       </c>
       <c r="G68" t="n">
-        <v>0.5590551181102362</v>
+        <v>4.503937007874016</v>
       </c>
       <c r="H68" t="n">
         <v>0</v>
       </c>
       <c r="I68" t="n">
-        <v>0</v>
-      </c>
-      <c r="J68" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J68" t="n">
+        <v>1</v>
+      </c>
       <c r="K68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L68" t="n">
         <v>0</v>
       </c>
       <c r="M68" t="n">
-        <v>0.1428571428571428</v>
+        <v>0.3103448275862069</v>
       </c>
       <c r="N68" t="n">
-        <v>0.0025177001953125</v>
+        <v>31.64771699905396</v>
       </c>
       <c r="O68" t="n">
-        <v>1122.97265625</v>
+        <v>1128.37109375</v>
       </c>
       <c r="P68" t="n">
-        <v>0</v>
+        <v>11.5</v>
       </c>
       <c r="Q68" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R68" t="n">
         <v>0</v>
@@ -4884,7 +5018,7 @@
         <v>0</v>
       </c>
       <c r="T68" t="n">
-        <v>0.002516746520996094</v>
+        <v>31.64771461486816</v>
       </c>
       <c r="U68" t="n">
         <v>0</v>

</xml_diff>